<commit_message>
docs: arquitetura em camadas, contrato da API e implantação com a decisão
- Diagrama de implantação com a escolha do Plano de Integração v2.3: ambiente
  integrado (Vercel, Render, Neon) e ambiente local (Docker Compose); sai a
  página da VM; legenda e situação da publicação explícitas
- docs/arquitetura/arquitetura-em-camadas.md (e PDF): camadas do site e da
  API, caminho de uma requisição, segurança, dados e decisões (HT03)
- Contrato da API legível (HTML e PDF): 51 operações com quem pode usar,
  corpo, resposta e os códigos observados na suíte (coleta_status.py)
- test_rotas_restantes.py: as 7 operações que nenhum teste chamava
- Relatório de execução refeito: 122 execuções em SQLite e PostgreSQL
</commit_message>
<xml_diff>
--- a/docs/testes/Relatorio_Execucao_Testes_SIGA_UEA.xlsx
+++ b/docs/testes/Relatorio_Execucao_Testes_SIGA_UEA.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Execucao por CT'!$A$1:$O$103</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Testes automatizados'!$A$1:$H$108</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Testes automatizados'!$A$1:$H$114</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Testes no navegador'!$A$1:$F$60</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Evidencias'!$A$1:$B$29</definedName>
   </definedNames>
@@ -602,7 +602,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>20/10/2026 20:31 (America/Manaus)</t>
+          <t>20/10/2026 21:01 (America/Manaus)</t>
         </is>
       </c>
     </row>
@@ -614,7 +614,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>c72c51c · branch dev · repositório SIGA-UEA/sigauea</t>
+          <t>449f0e6 · branch dev · repositório SIGA-UEA/sigauea</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B18" s="8">
-        <f>COUNTIF('Testes automatizados'!$E$2:$E$108,"Aprovado")</f>
+        <f>COUNTIF('Testes automatizados'!$E$2:$E$114,"Aprovado")</f>
         <v/>
       </c>
     </row>
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="B19" s="8">
-        <f>COUNTIF('Testes automatizados'!$E$2:$E$108,"Pulado")</f>
+        <f>COUNTIF('Testes automatizados'!$E$2:$E$114,"Pulado")</f>
         <v/>
       </c>
     </row>
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B20" s="8">
-        <f>COUNTIF('Testes automatizados'!$E$2:$E$108,"Reprovado")</f>
+        <f>COUNTIF('Testes automatizados'!$E$2:$E$114,"Reprovado")</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B21" s="8">
-        <f>COUNTIF('Testes automatizados'!$G$2:$G$108,"Aprovado")</f>
+        <f>COUNTIF('Testes automatizados'!$G$2:$G$114,"Aprovado")</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B22" s="8">
-        <f>COUNTIF('Testes automatizados'!$G$2:$G$108,"Pulado")</f>
+        <f>COUNTIF('Testes automatizados'!$G$2:$G$114,"Pulado")</f>
         <v/>
       </c>
     </row>
@@ -801,7 +801,7 @@
         </is>
       </c>
       <c r="B23" s="8">
-        <f>COUNTIF('Testes automatizados'!$G$2:$G$108,"Reprovado")</f>
+        <f>COUNTIF('Testes automatizados'!$G$2:$G$114,"Reprovado")</f>
         <v/>
       </c>
     </row>
@@ -852,7 +852,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Funções de teste da API: 107 (116 execuções contando os parâmetros). Um teste pulado é um caso Pendente na matriz: a funcionalidade ainda não existe (CT-01.10-06 depende do módulo de ideias; CT-06.01-04, da troca de orientador pela coordenação).</t>
+          <t>Funções de teste da API: 113 (122 execuções contando os parâmetros). Um teste pulado é um caso Pendente na matriz: a funcionalidade ainda não existe (CT-01.10-06 depende do módulo de ideias; CT-06.01-04, da troca de orientador pela coordenação).</t>
         </is>
       </c>
     </row>
@@ -9392,7 +9392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H108"/>
+  <dimension ref="A1:H114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -9472,7 +9472,7 @@
         </is>
       </c>
       <c r="F2" s="14" t="n">
-        <v>0.841</v>
+        <v>1.128</v>
       </c>
       <c r="G2" s="14" t="inlineStr">
         <is>
@@ -9480,7 +9480,7 @@
         </is>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.789</v>
+        <v>0.966</v>
       </c>
     </row>
     <row r="3">
@@ -9508,7 +9508,7 @@
         </is>
       </c>
       <c r="F3" s="14" t="n">
-        <v>4.09</v>
+        <v>4.388</v>
       </c>
       <c r="G3" s="14" t="inlineStr">
         <is>
@@ -9516,7 +9516,7 @@
         </is>
       </c>
       <c r="H3" s="14" t="n">
-        <v>3.574</v>
+        <v>3.963</v>
       </c>
     </row>
     <row r="4">
@@ -9544,7 +9544,7 @@
         </is>
       </c>
       <c r="F4" s="14" t="n">
-        <v>0.68</v>
+        <v>0.889</v>
       </c>
       <c r="G4" s="14" t="inlineStr">
         <is>
@@ -9552,7 +9552,7 @@
         </is>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.606</v>
+        <v>0.849</v>
       </c>
     </row>
     <row r="5">
@@ -9580,7 +9580,7 @@
         </is>
       </c>
       <c r="F5" s="14" t="n">
-        <v>0.8070000000000001</v>
+        <v>1.016</v>
       </c>
       <c r="G5" s="14" t="inlineStr">
         <is>
@@ -9588,7 +9588,7 @@
         </is>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.776</v>
+        <v>0.9330000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -9616,7 +9616,7 @@
         </is>
       </c>
       <c r="F6" s="14" t="n">
-        <v>1.143</v>
+        <v>1.106</v>
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
@@ -9624,7 +9624,7 @@
         </is>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.552</v>
+        <v>0.748</v>
       </c>
     </row>
     <row r="7">
@@ -9652,7 +9652,7 @@
         </is>
       </c>
       <c r="F7" s="14" t="n">
-        <v>0.93</v>
+        <v>0.944</v>
       </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
@@ -9660,7 +9660,7 @@
         </is>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.983</v>
+        <v>0.871</v>
       </c>
     </row>
     <row r="8">
@@ -9688,7 +9688,7 @@
         </is>
       </c>
       <c r="F8" s="14" t="n">
-        <v>1.016</v>
+        <v>0.946</v>
       </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
@@ -9696,7 +9696,7 @@
         </is>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.711</v>
+        <v>0.829</v>
       </c>
     </row>
     <row r="9">
@@ -9724,7 +9724,7 @@
         </is>
       </c>
       <c r="F9" s="14" t="n">
-        <v>0.776</v>
+        <v>0.71</v>
       </c>
       <c r="G9" s="14" t="inlineStr">
         <is>
@@ -9732,7 +9732,7 @@
         </is>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.577</v>
+        <v>0.709</v>
       </c>
     </row>
     <row r="10">
@@ -9760,7 +9760,7 @@
         </is>
       </c>
       <c r="F10" s="14" t="n">
-        <v>0.6919999999999999</v>
+        <v>0.781</v>
       </c>
       <c r="G10" s="14" t="inlineStr">
         <is>
@@ -9768,7 +9768,7 @@
         </is>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.653</v>
+        <v>0.794</v>
       </c>
     </row>
     <row r="11">
@@ -9796,7 +9796,7 @@
         </is>
       </c>
       <c r="F11" s="14" t="n">
-        <v>0.944</v>
+        <v>0.986</v>
       </c>
       <c r="G11" s="14" t="inlineStr">
         <is>
@@ -9804,7 +9804,7 @@
         </is>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.9340000000000001</v>
+        <v>1.033</v>
       </c>
     </row>
     <row r="12">
@@ -9832,7 +9832,7 @@
         </is>
       </c>
       <c r="F12" s="14" t="n">
-        <v>1.049</v>
+        <v>0.764</v>
       </c>
       <c r="G12" s="14" t="inlineStr">
         <is>
@@ -9840,7 +9840,7 @@
         </is>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.622</v>
+        <v>0.736</v>
       </c>
     </row>
     <row r="13">
@@ -9868,7 +9868,7 @@
         </is>
       </c>
       <c r="F13" s="14" t="n">
-        <v>0.633</v>
+        <v>0.6879999999999999</v>
       </c>
       <c r="G13" s="14" t="inlineStr">
         <is>
@@ -9876,7 +9876,7 @@
         </is>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.53</v>
+        <v>0.618</v>
       </c>
     </row>
     <row r="14">
@@ -9904,7 +9904,7 @@
         </is>
       </c>
       <c r="F14" s="14" t="n">
-        <v>1.227</v>
+        <v>1.589</v>
       </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
@@ -9912,7 +9912,7 @@
         </is>
       </c>
       <c r="H14" s="14" t="n">
-        <v>1.041</v>
+        <v>1.218</v>
       </c>
     </row>
     <row r="15">
@@ -9940,7 +9940,7 @@
         </is>
       </c>
       <c r="F15" s="14" t="n">
-        <v>0.672</v>
+        <v>0.719</v>
       </c>
       <c r="G15" s="14" t="inlineStr">
         <is>
@@ -9948,7 +9948,7 @@
         </is>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.622</v>
+        <v>0.875</v>
       </c>
     </row>
     <row r="16">
@@ -9976,7 +9976,7 @@
         </is>
       </c>
       <c r="F16" s="14" t="n">
-        <v>0.668</v>
+        <v>0.729</v>
       </c>
       <c r="G16" s="14" t="inlineStr">
         <is>
@@ -9984,7 +9984,7 @@
         </is>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.826</v>
+        <v>0.623</v>
       </c>
     </row>
     <row r="17">
@@ -10012,7 +10012,7 @@
         </is>
       </c>
       <c r="F17" s="14" t="n">
-        <v>1.079</v>
+        <v>0.752</v>
       </c>
       <c r="G17" s="14" t="inlineStr">
         <is>
@@ -10020,7 +10020,7 @@
         </is>
       </c>
       <c r="H17" s="14" t="n">
-        <v>0.672</v>
+        <v>0.994</v>
       </c>
     </row>
     <row r="18">
@@ -10048,7 +10048,7 @@
         </is>
       </c>
       <c r="F18" s="14" t="n">
-        <v>0.787</v>
+        <v>0.974</v>
       </c>
       <c r="G18" s="14" t="inlineStr">
         <is>
@@ -10056,7 +10056,7 @@
         </is>
       </c>
       <c r="H18" s="14" t="n">
-        <v>1.508</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="19">
@@ -10084,7 +10084,7 @@
         </is>
       </c>
       <c r="F19" s="14" t="n">
-        <v>0.876</v>
+        <v>1.27</v>
       </c>
       <c r="G19" s="14" t="inlineStr">
         <is>
@@ -10092,7 +10092,7 @@
         </is>
       </c>
       <c r="H19" s="14" t="n">
-        <v>0.696</v>
+        <v>0.86</v>
       </c>
     </row>
     <row r="20">
@@ -10120,7 +10120,7 @@
         </is>
       </c>
       <c r="F20" s="14" t="n">
-        <v>1.286</v>
+        <v>0.856</v>
       </c>
       <c r="G20" s="14" t="inlineStr">
         <is>
@@ -10128,7 +10128,7 @@
         </is>
       </c>
       <c r="H20" s="14" t="n">
-        <v>0.83</v>
+        <v>0.743</v>
       </c>
     </row>
     <row r="21">
@@ -10156,7 +10156,7 @@
         </is>
       </c>
       <c r="F21" s="14" t="n">
-        <v>2.36</v>
+        <v>2.576</v>
       </c>
       <c r="G21" s="14" t="inlineStr">
         <is>
@@ -10164,7 +10164,7 @@
         </is>
       </c>
       <c r="H21" s="14" t="n">
-        <v>2.615</v>
+        <v>2.397</v>
       </c>
     </row>
     <row r="22">
@@ -10192,7 +10192,7 @@
         </is>
       </c>
       <c r="F22" s="14" t="n">
-        <v>0.751</v>
+        <v>1.171</v>
       </c>
       <c r="G22" s="14" t="inlineStr">
         <is>
@@ -10200,7 +10200,7 @@
         </is>
       </c>
       <c r="H22" s="14" t="n">
-        <v>0.863</v>
+        <v>0.896</v>
       </c>
     </row>
     <row r="23">
@@ -10228,7 +10228,7 @@
         </is>
       </c>
       <c r="F23" s="14" t="n">
-        <v>0.661</v>
+        <v>0.741</v>
       </c>
       <c r="G23" s="14" t="inlineStr">
         <is>
@@ -10236,7 +10236,7 @@
         </is>
       </c>
       <c r="H23" s="14" t="n">
-        <v>0.535</v>
+        <v>0.869</v>
       </c>
     </row>
     <row r="24">
@@ -10264,7 +10264,7 @@
         </is>
       </c>
       <c r="F24" s="14" t="n">
-        <v>0.753</v>
+        <v>0.783</v>
       </c>
       <c r="G24" s="14" t="inlineStr">
         <is>
@@ -10272,7 +10272,7 @@
         </is>
       </c>
       <c r="H24" s="14" t="n">
-        <v>0.737</v>
+        <v>0.793</v>
       </c>
     </row>
     <row r="25">
@@ -10300,7 +10300,7 @@
         </is>
       </c>
       <c r="F25" s="14" t="n">
-        <v>0.744</v>
+        <v>0.79</v>
       </c>
       <c r="G25" s="14" t="inlineStr">
         <is>
@@ -10308,7 +10308,7 @@
         </is>
       </c>
       <c r="H25" s="14" t="n">
-        <v>0.737</v>
+        <v>0.839</v>
       </c>
     </row>
     <row r="26">
@@ -10336,7 +10336,7 @@
         </is>
       </c>
       <c r="F26" s="14" t="n">
-        <v>1.494</v>
+        <v>1.04</v>
       </c>
       <c r="G26" s="14" t="inlineStr">
         <is>
@@ -10344,7 +10344,7 @@
         </is>
       </c>
       <c r="H26" s="14" t="n">
-        <v>0.858</v>
+        <v>1.13</v>
       </c>
     </row>
     <row r="27">
@@ -10372,7 +10372,7 @@
         </is>
       </c>
       <c r="F27" s="14" t="n">
-        <v>0.5580000000000001</v>
+        <v>0.571</v>
       </c>
       <c r="G27" s="14" t="inlineStr">
         <is>
@@ -10380,7 +10380,7 @@
         </is>
       </c>
       <c r="H27" s="14" t="n">
-        <v>0.502</v>
+        <v>0.53</v>
       </c>
     </row>
     <row r="28">
@@ -10408,7 +10408,7 @@
         </is>
       </c>
       <c r="F28" s="14" t="n">
-        <v>1.001</v>
+        <v>1.572</v>
       </c>
       <c r="G28" s="14" t="inlineStr">
         <is>
@@ -10416,7 +10416,7 @@
         </is>
       </c>
       <c r="H28" s="14" t="n">
-        <v>1.283</v>
+        <v>1.085</v>
       </c>
     </row>
     <row r="29">
@@ -10444,7 +10444,7 @@
         </is>
       </c>
       <c r="F29" s="14" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="G29" s="14" t="inlineStr">
         <is>
@@ -10480,7 +10480,7 @@
         </is>
       </c>
       <c r="F30" s="14" t="n">
-        <v>2.875</v>
+        <v>2.603</v>
       </c>
       <c r="G30" s="14" t="inlineStr">
         <is>
@@ -10488,7 +10488,7 @@
         </is>
       </c>
       <c r="H30" s="14" t="n">
-        <v>1.637</v>
+        <v>2.11</v>
       </c>
     </row>
     <row r="31">
@@ -10516,7 +10516,7 @@
         </is>
       </c>
       <c r="F31" s="14" t="n">
-        <v>1.612</v>
+        <v>2.092</v>
       </c>
       <c r="G31" s="14" t="inlineStr">
         <is>
@@ -10524,7 +10524,7 @@
         </is>
       </c>
       <c r="H31" s="14" t="n">
-        <v>1.401</v>
+        <v>1.795</v>
       </c>
     </row>
     <row r="32">
@@ -10552,7 +10552,7 @@
         </is>
       </c>
       <c r="F32" s="14" t="n">
-        <v>1.665</v>
+        <v>1.94</v>
       </c>
       <c r="G32" s="14" t="inlineStr">
         <is>
@@ -10560,7 +10560,7 @@
         </is>
       </c>
       <c r="H32" s="14" t="n">
-        <v>1.97</v>
+        <v>1.782</v>
       </c>
     </row>
     <row r="33">
@@ -10588,7 +10588,7 @@
         </is>
       </c>
       <c r="F33" s="14" t="n">
-        <v>2.172</v>
+        <v>2.929</v>
       </c>
       <c r="G33" s="14" t="inlineStr">
         <is>
@@ -10596,7 +10596,7 @@
         </is>
       </c>
       <c r="H33" s="14" t="n">
-        <v>2.213</v>
+        <v>2.108</v>
       </c>
     </row>
     <row r="34">
@@ -10624,7 +10624,7 @@
         </is>
       </c>
       <c r="F34" s="14" t="n">
-        <v>5.038</v>
+        <v>6.11</v>
       </c>
       <c r="G34" s="14" t="inlineStr">
         <is>
@@ -10632,7 +10632,7 @@
         </is>
       </c>
       <c r="H34" s="14" t="n">
-        <v>4.579</v>
+        <v>4.898</v>
       </c>
     </row>
     <row r="35">
@@ -10660,7 +10660,7 @@
         </is>
       </c>
       <c r="F35" s="14" t="n">
-        <v>1.457</v>
+        <v>1.875</v>
       </c>
       <c r="G35" s="14" t="inlineStr">
         <is>
@@ -10668,7 +10668,7 @@
         </is>
       </c>
       <c r="H35" s="14" t="n">
-        <v>1.572</v>
+        <v>1.75</v>
       </c>
     </row>
     <row r="36">
@@ -10696,7 +10696,7 @@
         </is>
       </c>
       <c r="F36" s="14" t="n">
-        <v>1.522</v>
+        <v>2.107</v>
       </c>
       <c r="G36" s="14" t="inlineStr">
         <is>
@@ -10704,7 +10704,7 @@
         </is>
       </c>
       <c r="H36" s="14" t="n">
-        <v>1.719</v>
+        <v>1.918</v>
       </c>
     </row>
     <row r="37">
@@ -10732,15 +10732,15 @@
         </is>
       </c>
       <c r="F37" s="14" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G37" s="14" t="inlineStr">
+        <is>
+          <t>Pulado</t>
+        </is>
+      </c>
+      <c r="H37" s="14" t="n">
         <v>0</v>
-      </c>
-      <c r="G37" s="14" t="inlineStr">
-        <is>
-          <t>Pulado</t>
-        </is>
-      </c>
-      <c r="H37" s="14" t="n">
-        <v>0.001</v>
       </c>
     </row>
     <row r="38">
@@ -10768,7 +10768,7 @@
         </is>
       </c>
       <c r="F38" s="14" t="n">
-        <v>1.958</v>
+        <v>3.466</v>
       </c>
       <c r="G38" s="14" t="inlineStr">
         <is>
@@ -10776,7 +10776,7 @@
         </is>
       </c>
       <c r="H38" s="14" t="n">
-        <v>1.844</v>
+        <v>2.416</v>
       </c>
     </row>
     <row r="39">
@@ -10804,7 +10804,7 @@
         </is>
       </c>
       <c r="F39" s="14" t="n">
-        <v>1.928</v>
+        <v>2.638</v>
       </c>
       <c r="G39" s="14" t="inlineStr">
         <is>
@@ -10812,7 +10812,7 @@
         </is>
       </c>
       <c r="H39" s="14" t="n">
-        <v>1.698</v>
+        <v>2.022</v>
       </c>
     </row>
     <row r="40">
@@ -10840,7 +10840,7 @@
         </is>
       </c>
       <c r="F40" s="14" t="n">
-        <v>0.891</v>
+        <v>1.086</v>
       </c>
       <c r="G40" s="14" t="inlineStr">
         <is>
@@ -10848,7 +10848,7 @@
         </is>
       </c>
       <c r="H40" s="14" t="n">
-        <v>0.867</v>
+        <v>0.804</v>
       </c>
     </row>
     <row r="41">
@@ -10876,7 +10876,7 @@
         </is>
       </c>
       <c r="F41" s="14" t="n">
-        <v>1.675</v>
+        <v>1.683</v>
       </c>
       <c r="G41" s="14" t="inlineStr">
         <is>
@@ -10884,7 +10884,7 @@
         </is>
       </c>
       <c r="H41" s="14" t="n">
-        <v>0.884</v>
+        <v>1.201</v>
       </c>
     </row>
     <row r="42">
@@ -10912,7 +10912,7 @@
         </is>
       </c>
       <c r="F42" s="14" t="n">
-        <v>1.222</v>
+        <v>1.425</v>
       </c>
       <c r="G42" s="14" t="inlineStr">
         <is>
@@ -10920,7 +10920,7 @@
         </is>
       </c>
       <c r="H42" s="14" t="n">
-        <v>1.014</v>
+        <v>1.388</v>
       </c>
     </row>
     <row r="43">
@@ -10948,7 +10948,7 @@
         </is>
       </c>
       <c r="F43" s="14" t="n">
-        <v>1.196</v>
+        <v>1.329</v>
       </c>
       <c r="G43" s="14" t="inlineStr">
         <is>
@@ -10956,7 +10956,7 @@
         </is>
       </c>
       <c r="H43" s="14" t="n">
-        <v>1.304</v>
+        <v>1.047</v>
       </c>
     </row>
     <row r="44">
@@ -10984,7 +10984,7 @@
         </is>
       </c>
       <c r="F44" s="14" t="n">
-        <v>1.339</v>
+        <v>1.31</v>
       </c>
       <c r="G44" s="14" t="inlineStr">
         <is>
@@ -10992,7 +10992,7 @@
         </is>
       </c>
       <c r="H44" s="14" t="n">
-        <v>1.046</v>
+        <v>1.226</v>
       </c>
     </row>
     <row r="45">
@@ -11020,7 +11020,7 @@
         </is>
       </c>
       <c r="F45" s="14" t="n">
-        <v>1.055</v>
+        <v>1.69</v>
       </c>
       <c r="G45" s="14" t="inlineStr">
         <is>
@@ -11028,7 +11028,7 @@
         </is>
       </c>
       <c r="H45" s="14" t="n">
-        <v>1.235</v>
+        <v>1.327</v>
       </c>
     </row>
     <row r="46">
@@ -11056,7 +11056,7 @@
         </is>
       </c>
       <c r="F46" s="14" t="n">
-        <v>1.641</v>
+        <v>1.807</v>
       </c>
       <c r="G46" s="14" t="inlineStr">
         <is>
@@ -11064,7 +11064,7 @@
         </is>
       </c>
       <c r="H46" s="14" t="n">
-        <v>1.35</v>
+        <v>1.736</v>
       </c>
     </row>
     <row r="47">
@@ -11092,7 +11092,7 @@
         </is>
       </c>
       <c r="F47" s="14" t="n">
-        <v>1.132</v>
+        <v>1.114</v>
       </c>
       <c r="G47" s="14" t="inlineStr">
         <is>
@@ -11100,7 +11100,7 @@
         </is>
       </c>
       <c r="H47" s="14" t="n">
-        <v>1.459</v>
+        <v>0.984</v>
       </c>
     </row>
     <row r="48">
@@ -11128,7 +11128,7 @@
         </is>
       </c>
       <c r="F48" s="14" t="n">
-        <v>0.617</v>
+        <v>0.952</v>
       </c>
       <c r="G48" s="14" t="inlineStr">
         <is>
@@ -11136,7 +11136,7 @@
         </is>
       </c>
       <c r="H48" s="14" t="n">
-        <v>1.21</v>
+        <v>0.766</v>
       </c>
     </row>
     <row r="49">
@@ -11164,7 +11164,7 @@
         </is>
       </c>
       <c r="F49" s="14" t="n">
-        <v>0.8129999999999999</v>
+        <v>1.146</v>
       </c>
       <c r="G49" s="14" t="inlineStr">
         <is>
@@ -11172,7 +11172,7 @@
         </is>
       </c>
       <c r="H49" s="14" t="n">
-        <v>0.947</v>
+        <v>0.885</v>
       </c>
     </row>
     <row r="50">
@@ -11200,7 +11200,7 @@
         </is>
       </c>
       <c r="F50" s="14" t="n">
-        <v>0.954</v>
+        <v>1.424</v>
       </c>
       <c r="G50" s="14" t="inlineStr">
         <is>
@@ -11208,7 +11208,7 @@
         </is>
       </c>
       <c r="H50" s="14" t="n">
-        <v>1.424</v>
+        <v>1.055</v>
       </c>
     </row>
     <row r="51">
@@ -11236,7 +11236,7 @@
         </is>
       </c>
       <c r="F51" s="14" t="n">
-        <v>1.121</v>
+        <v>1.717</v>
       </c>
       <c r="G51" s="14" t="inlineStr">
         <is>
@@ -11244,7 +11244,7 @@
         </is>
       </c>
       <c r="H51" s="14" t="n">
-        <v>1.019</v>
+        <v>1.226</v>
       </c>
     </row>
     <row r="52">
@@ -11272,7 +11272,7 @@
         </is>
       </c>
       <c r="F52" s="14" t="n">
-        <v>1.138</v>
+        <v>1.631</v>
       </c>
       <c r="G52" s="14" t="inlineStr">
         <is>
@@ -11280,7 +11280,7 @@
         </is>
       </c>
       <c r="H52" s="14" t="n">
-        <v>1.058</v>
+        <v>1.071</v>
       </c>
     </row>
     <row r="53">
@@ -11308,7 +11308,7 @@
         </is>
       </c>
       <c r="F53" s="14" t="n">
-        <v>0.847</v>
+        <v>1.375</v>
       </c>
       <c r="G53" s="14" t="inlineStr">
         <is>
@@ -11316,7 +11316,7 @@
         </is>
       </c>
       <c r="H53" s="14" t="n">
-        <v>0.859</v>
+        <v>0.9379999999999999</v>
       </c>
     </row>
     <row r="54">
@@ -11344,7 +11344,7 @@
         </is>
       </c>
       <c r="F54" s="14" t="n">
-        <v>0.96</v>
+        <v>1.451</v>
       </c>
       <c r="G54" s="14" t="inlineStr">
         <is>
@@ -11352,7 +11352,7 @@
         </is>
       </c>
       <c r="H54" s="14" t="n">
-        <v>0.954</v>
+        <v>1.003</v>
       </c>
     </row>
     <row r="55">
@@ -11380,7 +11380,7 @@
         </is>
       </c>
       <c r="F55" s="14" t="n">
-        <v>0.803</v>
+        <v>1.436</v>
       </c>
       <c r="G55" s="14" t="inlineStr">
         <is>
@@ -11388,7 +11388,7 @@
         </is>
       </c>
       <c r="H55" s="14" t="n">
-        <v>1.018</v>
+        <v>0.983</v>
       </c>
     </row>
     <row r="56">
@@ -11416,7 +11416,7 @@
         </is>
       </c>
       <c r="F56" s="14" t="n">
-        <v>0.946</v>
+        <v>1.481</v>
       </c>
       <c r="G56" s="14" t="inlineStr">
         <is>
@@ -11424,7 +11424,7 @@
         </is>
       </c>
       <c r="H56" s="14" t="n">
-        <v>1.009</v>
+        <v>1.156</v>
       </c>
     </row>
     <row r="57">
@@ -11452,7 +11452,7 @@
         </is>
       </c>
       <c r="F57" s="14" t="n">
-        <v>0.925</v>
+        <v>1.426</v>
       </c>
       <c r="G57" s="14" t="inlineStr">
         <is>
@@ -11460,7 +11460,7 @@
         </is>
       </c>
       <c r="H57" s="14" t="n">
-        <v>1.196</v>
+        <v>1.098</v>
       </c>
     </row>
     <row r="58">
@@ -11488,7 +11488,7 @@
         </is>
       </c>
       <c r="F58" s="14" t="n">
-        <v>1.151</v>
+        <v>1.401</v>
       </c>
       <c r="G58" s="14" t="inlineStr">
         <is>
@@ -11496,7 +11496,7 @@
         </is>
       </c>
       <c r="H58" s="14" t="n">
-        <v>0.964</v>
+        <v>1.332</v>
       </c>
     </row>
     <row r="59">
@@ -11524,7 +11524,7 @@
         </is>
       </c>
       <c r="F59" s="14" t="n">
-        <v>0.867</v>
+        <v>1.429</v>
       </c>
       <c r="G59" s="14" t="inlineStr">
         <is>
@@ -11532,7 +11532,7 @@
         </is>
       </c>
       <c r="H59" s="14" t="n">
-        <v>1.105</v>
+        <v>1.33</v>
       </c>
     </row>
     <row r="60">
@@ -11560,7 +11560,7 @@
         </is>
       </c>
       <c r="F60" s="14" t="n">
-        <v>0.894</v>
+        <v>1.386</v>
       </c>
       <c r="G60" s="14" t="inlineStr">
         <is>
@@ -11568,7 +11568,7 @@
         </is>
       </c>
       <c r="H60" s="14" t="n">
-        <v>1.293</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="61">
@@ -11596,7 +11596,7 @@
         </is>
       </c>
       <c r="F61" s="14" t="n">
-        <v>0.707</v>
+        <v>1.221</v>
       </c>
       <c r="G61" s="14" t="inlineStr">
         <is>
@@ -11604,7 +11604,7 @@
         </is>
       </c>
       <c r="H61" s="14" t="n">
-        <v>0.848</v>
+        <v>0.844</v>
       </c>
     </row>
     <row r="62">
@@ -11632,7 +11632,7 @@
         </is>
       </c>
       <c r="F62" s="14" t="n">
-        <v>0.975</v>
+        <v>1.537</v>
       </c>
       <c r="G62" s="14" t="inlineStr">
         <is>
@@ -11640,7 +11640,7 @@
         </is>
       </c>
       <c r="H62" s="14" t="n">
-        <v>0.976</v>
+        <v>1.044</v>
       </c>
     </row>
     <row r="63">
@@ -11668,7 +11668,7 @@
         </is>
       </c>
       <c r="F63" s="14" t="n">
-        <v>1.968</v>
+        <v>2.498</v>
       </c>
       <c r="G63" s="14" t="inlineStr">
         <is>
@@ -11676,7 +11676,7 @@
         </is>
       </c>
       <c r="H63" s="14" t="n">
-        <v>1.533</v>
+        <v>1.612</v>
       </c>
     </row>
     <row r="64">
@@ -11704,7 +11704,7 @@
         </is>
       </c>
       <c r="F64" s="14" t="n">
-        <v>1.033</v>
+        <v>1.153</v>
       </c>
       <c r="G64" s="14" t="inlineStr">
         <is>
@@ -11712,18 +11712,18 @@
         </is>
       </c>
       <c r="H64" s="14" t="n">
-        <v>0.695</v>
+        <v>0.739</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="14" t="inlineStr">
         <is>
-          <t>test_tcc.py</t>
+          <t>test_rotas_restantes.py</t>
         </is>
       </c>
       <c r="B65" s="14" t="inlineStr">
         <is>
-          <t>test_ct_01_03_04_aluno_de_outro_curso_entra_e_mantem_o_curso</t>
+          <t>test_catalogo_de_cursos_e_perfis_exige_login</t>
         </is>
       </c>
       <c r="C65" s="14" t="n">
@@ -11731,7 +11731,7 @@
       </c>
       <c r="D65" s="14" t="inlineStr">
         <is>
-          <t>CT-01.03-04</t>
+          <t>complementar (sem CT na matriz)</t>
         </is>
       </c>
       <c r="E65" s="14" t="inlineStr">
@@ -11740,7 +11740,7 @@
         </is>
       </c>
       <c r="F65" s="14" t="n">
-        <v>1.556</v>
+        <v>0.977</v>
       </c>
       <c r="G65" s="14" t="inlineStr">
         <is>
@@ -11748,18 +11748,18 @@
         </is>
       </c>
       <c r="H65" s="14" t="n">
-        <v>1.843</v>
+        <v>0.716</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="14" t="inlineStr">
         <is>
-          <t>test_tcc.py</t>
+          <t>test_rotas_restantes.py</t>
         </is>
       </c>
       <c r="B66" s="14" t="inlineStr">
         <is>
-          <t>test_ct_03_01_01_formulario_traz_turma_orientadores_e_areas</t>
+          <t>test_coordenacao_remove_a_foto_do_docente</t>
         </is>
       </c>
       <c r="C66" s="14" t="n">
@@ -11767,7 +11767,7 @@
       </c>
       <c r="D66" s="14" t="inlineStr">
         <is>
-          <t>CT-03.01-01</t>
+          <t>complementar (sem CT na matriz)</t>
         </is>
       </c>
       <c r="E66" s="14" t="inlineStr">
@@ -11776,7 +11776,7 @@
         </is>
       </c>
       <c r="F66" s="14" t="n">
-        <v>1.388</v>
+        <v>1.109</v>
       </c>
       <c r="G66" s="14" t="inlineStr">
         <is>
@@ -11784,18 +11784,18 @@
         </is>
       </c>
       <c r="H66" s="14" t="n">
-        <v>1.615</v>
+        <v>1.947</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="14" t="inlineStr">
         <is>
-          <t>test_tcc.py</t>
+          <t>test_rotas_restantes.py</t>
         </is>
       </c>
       <c r="B67" s="14" t="inlineStr">
         <is>
-          <t>test_ct_03_01_02_e_03_01_03_resumo_ate_500_palavras_e_ate_10_palavras_chave</t>
+          <t>test_health_responde_sem_login</t>
         </is>
       </c>
       <c r="C67" s="14" t="n">
@@ -11803,7 +11803,7 @@
       </c>
       <c r="D67" s="14" t="inlineStr">
         <is>
-          <t>CT-03.01-02, CT-03.01-03</t>
+          <t>complementar (sem CT na matriz)</t>
         </is>
       </c>
       <c r="E67" s="14" t="inlineStr">
@@ -11812,7 +11812,7 @@
         </is>
       </c>
       <c r="F67" s="14" t="n">
-        <v>1.537</v>
+        <v>0.72</v>
       </c>
       <c r="G67" s="14" t="inlineStr">
         <is>
@@ -11820,18 +11820,18 @@
         </is>
       </c>
       <c r="H67" s="14" t="n">
-        <v>1.429</v>
+        <v>0.582</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="14" t="inlineStr">
         <is>
-          <t>test_tcc.py</t>
+          <t>test_rotas_restantes.py</t>
         </is>
       </c>
       <c r="B68" s="14" t="inlineStr">
         <is>
-          <t>test_ct_03_01_04_e_03_04_02_e_06_01_01_rascunho_sem_protocolo_e_vinculo_pendente</t>
+          <t>test_lista_de_periodos_e_de_turmas</t>
         </is>
       </c>
       <c r="C68" s="14" t="n">
@@ -11839,7 +11839,7 @@
       </c>
       <c r="D68" s="14" t="inlineStr">
         <is>
-          <t>CT-03.01-04, CT-03.01-05, CT-03.04-02, CT-06.01-01</t>
+          <t>complementar (sem CT na matriz)</t>
         </is>
       </c>
       <c r="E68" s="14" t="inlineStr">
@@ -11848,7 +11848,7 @@
         </is>
       </c>
       <c r="F68" s="14" t="n">
-        <v>1.675</v>
+        <v>2.828</v>
       </c>
       <c r="G68" s="14" t="inlineStr">
         <is>
@@ -11856,18 +11856,18 @@
         </is>
       </c>
       <c r="H68" s="14" t="n">
-        <v>1.474</v>
+        <v>1.744</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="14" t="inlineStr">
         <is>
-          <t>test_tcc.py</t>
+          <t>test_rotas_restantes.py</t>
         </is>
       </c>
       <c r="B69" s="14" t="inlineStr">
         <is>
-          <t>test_ct_03_01_08_editar_rascunho_audita_cada_campo</t>
+          <t>test_orientador_abre_a_solicitacao_e_outro_docente_nao</t>
         </is>
       </c>
       <c r="C69" s="14" t="n">
@@ -11875,7 +11875,7 @@
       </c>
       <c r="D69" s="14" t="inlineStr">
         <is>
-          <t>CT-03.01-08</t>
+          <t>complementar (sem CT na matriz)</t>
         </is>
       </c>
       <c r="E69" s="14" t="inlineStr">
@@ -11884,7 +11884,7 @@
         </is>
       </c>
       <c r="F69" s="14" t="n">
-        <v>1.537</v>
+        <v>2.898</v>
       </c>
       <c r="G69" s="14" t="inlineStr">
         <is>
@@ -11892,18 +11892,18 @@
         </is>
       </c>
       <c r="H69" s="14" t="n">
-        <v>1.583</v>
+        <v>2.131</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="14" t="inlineStr">
         <is>
-          <t>test_tcc.py</t>
+          <t>test_rotas_restantes.py</t>
         </is>
       </c>
       <c r="B70" s="14" t="inlineStr">
         <is>
-          <t>test_ct_03_02_03_e_03_02_04_artigo_publicado_exige_doi</t>
+          <t>test_so_a_coordenacao_remove_foto_de_outra_pessoa</t>
         </is>
       </c>
       <c r="C70" s="14" t="n">
@@ -11911,7 +11911,7 @@
       </c>
       <c r="D70" s="14" t="inlineStr">
         <is>
-          <t>CT-03.02-03, CT-03.02-04</t>
+          <t>complementar (sem CT na matriz)</t>
         </is>
       </c>
       <c r="E70" s="14" t="inlineStr">
@@ -11920,7 +11920,7 @@
         </is>
       </c>
       <c r="F70" s="14" t="n">
-        <v>1.72</v>
+        <v>2.754</v>
       </c>
       <c r="G70" s="14" t="inlineStr">
         <is>
@@ -11928,7 +11928,7 @@
         </is>
       </c>
       <c r="H70" s="14" t="n">
-        <v>1.708</v>
+        <v>3.522</v>
       </c>
     </row>
     <row r="71">
@@ -11939,7 +11939,7 @@
       </c>
       <c r="B71" s="14" t="inlineStr">
         <is>
-          <t>test_ct_03_03_01_e_03_03_06_e_03_04_01_submissao_gera_protocolo_unico_e_repetir_nao_duplica</t>
+          <t>test_ct_01_03_04_aluno_de_outro_curso_entra_e_mantem_o_curso</t>
         </is>
       </c>
       <c r="C71" s="14" t="n">
@@ -11947,7 +11947,7 @@
       </c>
       <c r="D71" s="14" t="inlineStr">
         <is>
-          <t>CT-03.03-01, CT-03.03-05, CT-03.03-06, CT-03.03-08, CT-03.04-01, CT-03.04-03, CT-03.04-06</t>
+          <t>CT-01.03-04</t>
         </is>
       </c>
       <c r="E71" s="14" t="inlineStr">
@@ -11956,7 +11956,7 @@
         </is>
       </c>
       <c r="F71" s="14" t="n">
-        <v>1.527</v>
+        <v>2.631</v>
       </c>
       <c r="G71" s="14" t="inlineStr">
         <is>
@@ -11964,7 +11964,7 @@
         </is>
       </c>
       <c r="H71" s="14" t="n">
-        <v>1.974</v>
+        <v>3.42</v>
       </c>
     </row>
     <row r="72">
@@ -11975,7 +11975,7 @@
       </c>
       <c r="B72" s="14" t="inlineStr">
         <is>
-          <t>test_ct_03_03_02_campos_obrigatorios</t>
+          <t>test_ct_03_01_01_formulario_traz_turma_orientadores_e_areas</t>
         </is>
       </c>
       <c r="C72" s="14" t="n">
@@ -11983,7 +11983,7 @@
       </c>
       <c r="D72" s="14" t="inlineStr">
         <is>
-          <t>CT-03.03-02</t>
+          <t>CT-03.01-01</t>
         </is>
       </c>
       <c r="E72" s="14" t="inlineStr">
@@ -11992,7 +11992,7 @@
         </is>
       </c>
       <c r="F72" s="14" t="n">
-        <v>1.924</v>
+        <v>2.094</v>
       </c>
       <c r="G72" s="14" t="inlineStr">
         <is>
@@ -12000,7 +12000,7 @@
         </is>
       </c>
       <c r="H72" s="14" t="n">
-        <v>1.851</v>
+        <v>2.017</v>
       </c>
     </row>
     <row r="73">
@@ -12011,7 +12011,7 @@
       </c>
       <c r="B73" s="14" t="inlineStr">
         <is>
-          <t>test_ct_03_03_03_desistente_nao_submete</t>
+          <t>test_ct_03_01_02_e_03_01_03_resumo_ate_500_palavras_e_ate_10_palavras_chave</t>
         </is>
       </c>
       <c r="C73" s="14" t="n">
@@ -12019,7 +12019,7 @@
       </c>
       <c r="D73" s="14" t="inlineStr">
         <is>
-          <t>CT-03.03-03</t>
+          <t>CT-03.01-02, CT-03.01-03</t>
         </is>
       </c>
       <c r="E73" s="14" t="inlineStr">
@@ -12028,7 +12028,7 @@
         </is>
       </c>
       <c r="F73" s="14" t="n">
-        <v>1.459</v>
+        <v>1.647</v>
       </c>
       <c r="G73" s="14" t="inlineStr">
         <is>
@@ -12036,7 +12036,7 @@
         </is>
       </c>
       <c r="H73" s="14" t="n">
-        <v>1.531</v>
+        <v>2.052</v>
       </c>
     </row>
     <row r="74">
@@ -12047,7 +12047,7 @@
       </c>
       <c r="B74" s="14" t="inlineStr">
         <is>
-          <t>test_ct_03_04_04_um_cadastro_por_periodo</t>
+          <t>test_ct_03_01_04_e_03_04_02_e_06_01_01_rascunho_sem_protocolo_e_vinculo_pendente</t>
         </is>
       </c>
       <c r="C74" s="14" t="n">
@@ -12055,7 +12055,7 @@
       </c>
       <c r="D74" s="14" t="inlineStr">
         <is>
-          <t>CT-03.04-04</t>
+          <t>CT-03.01-04, CT-03.01-05, CT-03.04-02, CT-06.01-01</t>
         </is>
       </c>
       <c r="E74" s="14" t="inlineStr">
@@ -12064,7 +12064,7 @@
         </is>
       </c>
       <c r="F74" s="14" t="n">
-        <v>1.4</v>
+        <v>1.901</v>
       </c>
       <c r="G74" s="14" t="inlineStr">
         <is>
@@ -12072,7 +12072,7 @@
         </is>
       </c>
       <c r="H74" s="14" t="n">
-        <v>1.439</v>
+        <v>2.198</v>
       </c>
     </row>
     <row r="75">
@@ -12083,7 +12083,7 @@
       </c>
       <c r="B75" s="14" t="inlineStr">
         <is>
-          <t>test_ds_fl01b_e2_orientador_nao_elegivel</t>
+          <t>test_ct_03_01_08_editar_rascunho_audita_cada_campo</t>
         </is>
       </c>
       <c r="C75" s="14" t="n">
@@ -12091,7 +12091,7 @@
       </c>
       <c r="D75" s="14" t="inlineStr">
         <is>
-          <t>complementar (sem CT na matriz)</t>
+          <t>CT-03.01-08</t>
         </is>
       </c>
       <c r="E75" s="14" t="inlineStr">
@@ -12100,7 +12100,7 @@
         </is>
       </c>
       <c r="F75" s="14" t="n">
-        <v>1.452</v>
+        <v>2.239</v>
       </c>
       <c r="G75" s="14" t="inlineStr">
         <is>
@@ -12108,7 +12108,7 @@
         </is>
       </c>
       <c r="H75" s="14" t="n">
-        <v>1.373</v>
+        <v>3.685</v>
       </c>
     </row>
     <row r="76">
@@ -12119,7 +12119,7 @@
       </c>
       <c r="B76" s="14" t="inlineStr">
         <is>
-          <t>test_ds_fl01b_em_analise_nao_edita</t>
+          <t>test_ct_03_02_03_e_03_02_04_artigo_publicado_exige_doi</t>
         </is>
       </c>
       <c r="C76" s="14" t="n">
@@ -12127,7 +12127,7 @@
       </c>
       <c r="D76" s="14" t="inlineStr">
         <is>
-          <t>complementar (sem CT na matriz)</t>
+          <t>CT-03.02-03, CT-03.02-04</t>
         </is>
       </c>
       <c r="E76" s="14" t="inlineStr">
@@ -12136,7 +12136,7 @@
         </is>
       </c>
       <c r="F76" s="14" t="n">
-        <v>1.5</v>
+        <v>2.236</v>
       </c>
       <c r="G76" s="14" t="inlineStr">
         <is>
@@ -12144,7 +12144,7 @@
         </is>
       </c>
       <c r="H76" s="14" t="n">
-        <v>1.673</v>
+        <v>3.65</v>
       </c>
     </row>
     <row r="77">
@@ -12155,7 +12155,7 @@
       </c>
       <c r="B77" s="14" t="inlineStr">
         <is>
-          <t>test_ds_fl03_orientador_aceita_e_aluno_e_avisado</t>
+          <t>test_ct_03_03_01_e_03_03_06_e_03_04_01_submissao_gera_protocolo_unico_e_repetir_nao_duplica</t>
         </is>
       </c>
       <c r="C77" s="14" t="n">
@@ -12163,7 +12163,7 @@
       </c>
       <c r="D77" s="14" t="inlineStr">
         <is>
-          <t>complementar (sem CT na matriz)</t>
+          <t>CT-03.03-01, CT-03.03-05, CT-03.03-06, CT-03.03-08, CT-03.04-01, CT-03.04-03, CT-03.04-06</t>
         </is>
       </c>
       <c r="E77" s="14" t="inlineStr">
@@ -12172,7 +12172,7 @@
         </is>
       </c>
       <c r="F77" s="14" t="n">
-        <v>2.032</v>
+        <v>2.427</v>
       </c>
       <c r="G77" s="14" t="inlineStr">
         <is>
@@ -12180,7 +12180,7 @@
         </is>
       </c>
       <c r="H77" s="14" t="n">
-        <v>1.719</v>
+        <v>2.276</v>
       </c>
     </row>
     <row r="78">
@@ -12191,7 +12191,7 @@
       </c>
       <c r="B78" s="14" t="inlineStr">
         <is>
-          <t>test_ds_fl03_recusa_exige_motivo_e_nao_pode_responder_duas_vezes</t>
+          <t>test_ct_03_03_02_campos_obrigatorios</t>
         </is>
       </c>
       <c r="C78" s="14" t="n">
@@ -12199,7 +12199,7 @@
       </c>
       <c r="D78" s="14" t="inlineStr">
         <is>
-          <t>complementar (sem CT na matriz)</t>
+          <t>CT-03.03-02</t>
         </is>
       </c>
       <c r="E78" s="14" t="inlineStr">
@@ -12208,7 +12208,7 @@
         </is>
       </c>
       <c r="F78" s="14" t="n">
-        <v>2.155</v>
+        <v>2.072</v>
       </c>
       <c r="G78" s="14" t="inlineStr">
         <is>
@@ -12216,7 +12216,7 @@
         </is>
       </c>
       <c r="H78" s="14" t="n">
-        <v>2.143</v>
+        <v>3.12</v>
       </c>
     </row>
     <row r="79">
@@ -12227,7 +12227,7 @@
       </c>
       <c r="B79" s="14" t="inlineStr">
         <is>
-          <t>test_ds_fl03b_apos_recusa_aluno_indica_outro_orientador</t>
+          <t>test_ct_03_03_03_desistente_nao_submete</t>
         </is>
       </c>
       <c r="C79" s="14" t="n">
@@ -12235,7 +12235,7 @@
       </c>
       <c r="D79" s="14" t="inlineStr">
         <is>
-          <t>complementar (sem CT na matriz)</t>
+          <t>CT-03.03-03</t>
         </is>
       </c>
       <c r="E79" s="14" t="inlineStr">
@@ -12244,7 +12244,7 @@
         </is>
       </c>
       <c r="F79" s="14" t="n">
-        <v>2.022</v>
+        <v>2.039</v>
       </c>
       <c r="G79" s="14" t="inlineStr">
         <is>
@@ -12252,7 +12252,7 @@
         </is>
       </c>
       <c r="H79" s="14" t="n">
-        <v>1.877</v>
+        <v>3.813</v>
       </c>
     </row>
     <row r="80">
@@ -12263,7 +12263,7 @@
       </c>
       <c r="B80" s="14" t="inlineStr">
         <is>
-          <t>test_minhas_turmas_do_aluno_mostra_matricula_e_o_proprio_tcc</t>
+          <t>test_ct_03_04_04_um_cadastro_por_periodo</t>
         </is>
       </c>
       <c r="C80" s="14" t="n">
@@ -12271,7 +12271,7 @@
       </c>
       <c r="D80" s="14" t="inlineStr">
         <is>
-          <t>complementar (sem CT na matriz)</t>
+          <t>CT-03.04-04</t>
         </is>
       </c>
       <c r="E80" s="14" t="inlineStr">
@@ -12280,7 +12280,7 @@
         </is>
       </c>
       <c r="F80" s="14" t="n">
-        <v>1.621</v>
+        <v>1.939</v>
       </c>
       <c r="G80" s="14" t="inlineStr">
         <is>
@@ -12288,7 +12288,7 @@
         </is>
       </c>
       <c r="H80" s="14" t="n">
-        <v>2.005</v>
+        <v>2.243</v>
       </c>
     </row>
     <row r="81">
@@ -12299,7 +12299,7 @@
       </c>
       <c r="B81" s="14" t="inlineStr">
         <is>
-          <t>test_minhas_turmas_do_professor_com_contagem_de_alunos_e_tccs</t>
+          <t>test_ds_fl01b_e2_orientador_nao_elegivel</t>
         </is>
       </c>
       <c r="C81" s="14" t="n">
@@ -12316,7 +12316,7 @@
         </is>
       </c>
       <c r="F81" s="14" t="n">
-        <v>2.081</v>
+        <v>2.094</v>
       </c>
       <c r="G81" s="14" t="inlineStr">
         <is>
@@ -12324,7 +12324,7 @@
         </is>
       </c>
       <c r="H81" s="14" t="n">
-        <v>1.939</v>
+        <v>2.777</v>
       </c>
     </row>
     <row r="82">
@@ -12335,7 +12335,7 @@
       </c>
       <c r="B82" s="14" t="inlineStr">
         <is>
-          <t>test_minhas_turmas_so_mostra_ao_docente_as_turmas_que_ele_conduz</t>
+          <t>test_ds_fl01b_em_analise_nao_edita</t>
         </is>
       </c>
       <c r="C82" s="14" t="n">
@@ -12352,7 +12352,7 @@
         </is>
       </c>
       <c r="F82" s="14" t="n">
-        <v>1.503</v>
+        <v>2.022</v>
       </c>
       <c r="G82" s="14" t="inlineStr">
         <is>
@@ -12360,7 +12360,7 @@
         </is>
       </c>
       <c r="H82" s="14" t="n">
-        <v>1.613</v>
+        <v>3.563</v>
       </c>
     </row>
     <row r="83">
@@ -12371,7 +12371,7 @@
       </c>
       <c r="B83" s="14" t="inlineStr">
         <is>
-          <t>test_rbn0303_nao_submete_sem_aceite_do_orientador</t>
+          <t>test_ds_fl03_orientador_aceita_e_aluno_e_avisado</t>
         </is>
       </c>
       <c r="C83" s="14" t="n">
@@ -12388,7 +12388,7 @@
         </is>
       </c>
       <c r="F83" s="14" t="n">
-        <v>1.654</v>
+        <v>2.228</v>
       </c>
       <c r="G83" s="14" t="inlineStr">
         <is>
@@ -12396,7 +12396,7 @@
         </is>
       </c>
       <c r="H83" s="14" t="n">
-        <v>2.012</v>
+        <v>3.724</v>
       </c>
     </row>
     <row r="84">
@@ -12407,7 +12407,7 @@
       </c>
       <c r="B84" s="14" t="inlineStr">
         <is>
-          <t>test_rbn0305_devolvido_e_corrigido_mantem_o_protocolo</t>
+          <t>test_ds_fl03_recusa_exige_motivo_e_nao_pode_responder_duas_vezes</t>
         </is>
       </c>
       <c r="C84" s="14" t="n">
@@ -12424,7 +12424,7 @@
         </is>
       </c>
       <c r="F84" s="14" t="n">
-        <v>2.018</v>
+        <v>2.613</v>
       </c>
       <c r="G84" s="14" t="inlineStr">
         <is>
@@ -12432,7 +12432,7 @@
         </is>
       </c>
       <c r="H84" s="14" t="n">
-        <v>1.639</v>
+        <v>3.499</v>
       </c>
     </row>
     <row r="85">
@@ -12443,7 +12443,7 @@
       </c>
       <c r="B85" s="14" t="inlineStr">
         <is>
-          <t>test_rbn0501_listas_por_perfil</t>
+          <t>test_ds_fl03b_apos_recusa_aluno_indica_outro_orientador</t>
         </is>
       </c>
       <c r="C85" s="14" t="n">
@@ -12460,7 +12460,7 @@
         </is>
       </c>
       <c r="F85" s="14" t="n">
-        <v>1.426</v>
+        <v>2.226</v>
       </c>
       <c r="G85" s="14" t="inlineStr">
         <is>
@@ -12468,7 +12468,7 @@
         </is>
       </c>
       <c r="H85" s="14" t="n">
-        <v>1.927</v>
+        <v>3.821</v>
       </c>
     </row>
     <row r="86">
@@ -12479,7 +12479,7 @@
       </c>
       <c r="B86" s="14" t="inlineStr">
         <is>
-          <t>test_rbn0801_so_a_coordenacao_cria_turma</t>
+          <t>test_minhas_turmas_do_aluno_mostra_matricula_e_o_proprio_tcc</t>
         </is>
       </c>
       <c r="C86" s="14" t="n">
@@ -12496,7 +12496,7 @@
         </is>
       </c>
       <c r="F86" s="14" t="n">
-        <v>1.427</v>
+        <v>2.075</v>
       </c>
       <c r="G86" s="14" t="inlineStr">
         <is>
@@ -12504,7 +12504,7 @@
         </is>
       </c>
       <c r="H86" s="14" t="n">
-        <v>1.625</v>
+        <v>3.024</v>
       </c>
     </row>
     <row r="87">
@@ -12515,7 +12515,7 @@
       </c>
       <c r="B87" s="14" t="inlineStr">
         <is>
-          <t>test_rbn0801_turma_criada_com_codigo_do_curso_e_periodo</t>
+          <t>test_minhas_turmas_do_professor_com_contagem_de_alunos_e_tccs</t>
         </is>
       </c>
       <c r="C87" s="14" t="n">
@@ -12532,7 +12532,7 @@
         </is>
       </c>
       <c r="F87" s="14" t="n">
-        <v>1.422</v>
+        <v>3.243</v>
       </c>
       <c r="G87" s="14" t="inlineStr">
         <is>
@@ -12540,7 +12540,7 @@
         </is>
       </c>
       <c r="H87" s="14" t="n">
-        <v>1.618</v>
+        <v>3.99</v>
       </c>
     </row>
     <row r="88">
@@ -12551,7 +12551,7 @@
       </c>
       <c r="B88" s="14" t="inlineStr">
         <is>
-          <t>test_rn05_aluno_sem_matricula_nao_abre_nem_salva</t>
+          <t>test_minhas_turmas_so_mostra_ao_docente_as_turmas_que_ele_conduz</t>
         </is>
       </c>
       <c r="C88" s="14" t="n">
@@ -12568,7 +12568,7 @@
         </is>
       </c>
       <c r="F88" s="14" t="n">
-        <v>1.601</v>
+        <v>2.342</v>
       </c>
       <c r="G88" s="14" t="inlineStr">
         <is>
@@ -12576,7 +12576,7 @@
         </is>
       </c>
       <c r="H88" s="14" t="n">
-        <v>1.584</v>
+        <v>3.284</v>
       </c>
     </row>
     <row r="89">
@@ -12587,7 +12587,7 @@
       </c>
       <c r="B89" s="14" t="inlineStr">
         <is>
-          <t>test_rn07_aluno_e_outro_docente_nao_abrem_a_turma</t>
+          <t>test_rbn0303_nao_submete_sem_aceite_do_orientador</t>
         </is>
       </c>
       <c r="C89" s="14" t="n">
@@ -12604,7 +12604,7 @@
         </is>
       </c>
       <c r="F89" s="14" t="n">
-        <v>1.709</v>
+        <v>2.594</v>
       </c>
       <c r="G89" s="14" t="inlineStr">
         <is>
@@ -12612,7 +12612,7 @@
         </is>
       </c>
       <c r="H89" s="14" t="n">
-        <v>1.569</v>
+        <v>3.205</v>
       </c>
     </row>
     <row r="90">
@@ -12623,7 +12623,7 @@
       </c>
       <c r="B90" s="14" t="inlineStr">
         <is>
-          <t>test_rn07_orientador_so_responde_os_proprios_pedidos</t>
+          <t>test_rbn0305_devolvido_e_corrigido_mantem_o_protocolo</t>
         </is>
       </c>
       <c r="C90" s="14" t="n">
@@ -12640,7 +12640,7 @@
         </is>
       </c>
       <c r="F90" s="14" t="n">
-        <v>1.581</v>
+        <v>2.352</v>
       </c>
       <c r="G90" s="14" t="inlineStr">
         <is>
@@ -12648,7 +12648,7 @@
         </is>
       </c>
       <c r="H90" s="14" t="n">
-        <v>2.318</v>
+        <v>4.102</v>
       </c>
     </row>
     <row r="91">
@@ -12659,7 +12659,7 @@
       </c>
       <c r="B91" s="14" t="inlineStr">
         <is>
-          <t>test_rn07_outro_aluno_nao_ve_nem_edita</t>
+          <t>test_rbn0501_listas_por_perfil</t>
         </is>
       </c>
       <c r="C91" s="14" t="n">
@@ -12676,7 +12676,7 @@
         </is>
       </c>
       <c r="F91" s="14" t="n">
-        <v>1.968</v>
+        <v>1.918</v>
       </c>
       <c r="G91" s="14" t="inlineStr">
         <is>
@@ -12684,18 +12684,18 @@
         </is>
       </c>
       <c r="H91" s="14" t="n">
-        <v>1.983</v>
+        <v>3.753</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="14" t="inlineStr">
         <is>
-          <t>test_usuarios.py</t>
+          <t>test_tcc.py</t>
         </is>
       </c>
       <c r="B92" s="14" t="inlineStr">
         <is>
-          <t>test_ct_01_01_01_docente_nasce_inativo_e_sem_senha</t>
+          <t>test_rbn0801_so_a_coordenacao_cria_turma</t>
         </is>
       </c>
       <c r="C92" s="14" t="n">
@@ -12703,7 +12703,7 @@
       </c>
       <c r="D92" s="14" t="inlineStr">
         <is>
-          <t>CT-01.01-01</t>
+          <t>complementar (sem CT na matriz)</t>
         </is>
       </c>
       <c r="E92" s="14" t="inlineStr">
@@ -12712,7 +12712,7 @@
         </is>
       </c>
       <c r="F92" s="14" t="n">
-        <v>0.604</v>
+        <v>2.523</v>
       </c>
       <c r="G92" s="14" t="inlineStr">
         <is>
@@ -12720,18 +12720,18 @@
         </is>
       </c>
       <c r="H92" s="14" t="n">
-        <v>0.612</v>
+        <v>3.468</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="14" t="inlineStr">
         <is>
-          <t>test_usuarios.py</t>
+          <t>test_tcc.py</t>
         </is>
       </c>
       <c r="B93" s="14" t="inlineStr">
         <is>
-          <t>test_ct_01_01_02_campo_obrigatorio_vazio_responde_400</t>
+          <t>test_rbn0801_turma_criada_com_codigo_do_curso_e_periodo</t>
         </is>
       </c>
       <c r="C93" s="14" t="n">
@@ -12739,7 +12739,7 @@
       </c>
       <c r="D93" s="14" t="inlineStr">
         <is>
-          <t>CT-01.01-02</t>
+          <t>complementar (sem CT na matriz)</t>
         </is>
       </c>
       <c r="E93" s="14" t="inlineStr">
@@ -12748,7 +12748,7 @@
         </is>
       </c>
       <c r="F93" s="14" t="n">
-        <v>0.5610000000000001</v>
+        <v>2.421</v>
       </c>
       <c r="G93" s="14" t="inlineStr">
         <is>
@@ -12756,18 +12756,18 @@
         </is>
       </c>
       <c r="H93" s="14" t="n">
-        <v>0.576</v>
+        <v>3.647</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="14" t="inlineStr">
         <is>
-          <t>test_usuarios.py</t>
+          <t>test_tcc.py</t>
         </is>
       </c>
       <c r="B94" s="14" t="inlineStr">
         <is>
-          <t>test_ct_01_01_03_email_duplicado_ignora_maiusculas</t>
+          <t>test_rn05_aluno_sem_matricula_nao_abre_nem_salva</t>
         </is>
       </c>
       <c r="C94" s="14" t="n">
@@ -12775,7 +12775,7 @@
       </c>
       <c r="D94" s="14" t="inlineStr">
         <is>
-          <t>CT-01.01-03</t>
+          <t>complementar (sem CT na matriz)</t>
         </is>
       </c>
       <c r="E94" s="14" t="inlineStr">
@@ -12784,7 +12784,7 @@
         </is>
       </c>
       <c r="F94" s="14" t="n">
-        <v>0.597</v>
+        <v>2.321</v>
       </c>
       <c r="G94" s="14" t="inlineStr">
         <is>
@@ -12792,18 +12792,18 @@
         </is>
       </c>
       <c r="H94" s="14" t="n">
-        <v>0.553</v>
+        <v>2.312</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="14" t="inlineStr">
         <is>
-          <t>test_usuarios.py</t>
+          <t>test_tcc.py</t>
         </is>
       </c>
       <c r="B95" s="14" t="inlineStr">
         <is>
-          <t>test_ct_01_01_05_coordenador_nao_exige_curso</t>
+          <t>test_rn07_aluno_e_outro_docente_nao_abrem_a_turma</t>
         </is>
       </c>
       <c r="C95" s="14" t="n">
@@ -12811,7 +12811,7 @@
       </c>
       <c r="D95" s="14" t="inlineStr">
         <is>
-          <t>CT-01.01-05</t>
+          <t>complementar (sem CT na matriz)</t>
         </is>
       </c>
       <c r="E95" s="14" t="inlineStr">
@@ -12820,7 +12820,7 @@
         </is>
       </c>
       <c r="F95" s="14" t="n">
-        <v>0.871</v>
+        <v>2.192</v>
       </c>
       <c r="G95" s="14" t="inlineStr">
         <is>
@@ -12828,18 +12828,18 @@
         </is>
       </c>
       <c r="H95" s="14" t="n">
-        <v>0.591</v>
+        <v>2.257</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="14" t="inlineStr">
         <is>
-          <t>test_usuarios.py</t>
+          <t>test_tcc.py</t>
         </is>
       </c>
       <c r="B96" s="14" t="inlineStr">
         <is>
-          <t>test_ct_01_01_06_quem_nao_e_coordenador_recebe_403</t>
+          <t>test_rn07_orientador_so_responde_os_proprios_pedidos</t>
         </is>
       </c>
       <c r="C96" s="14" t="n">
@@ -12847,7 +12847,7 @@
       </c>
       <c r="D96" s="14" t="inlineStr">
         <is>
-          <t>CT-01.01-06</t>
+          <t>complementar (sem CT na matriz)</t>
         </is>
       </c>
       <c r="E96" s="14" t="inlineStr">
@@ -12856,7 +12856,7 @@
         </is>
       </c>
       <c r="F96" s="14" t="n">
-        <v>0.823</v>
+        <v>2.141</v>
       </c>
       <c r="G96" s="14" t="inlineStr">
         <is>
@@ -12864,18 +12864,18 @@
         </is>
       </c>
       <c r="H96" s="14" t="n">
-        <v>0.789</v>
+        <v>4.23</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="14" t="inlineStr">
         <is>
-          <t>test_usuarios.py</t>
+          <t>test_tcc.py</t>
         </is>
       </c>
       <c r="B97" s="14" t="inlineStr">
         <is>
-          <t>test_ct_01_01_07_criacao_fica_no_log</t>
+          <t>test_rn07_outro_aluno_nao_ve_nem_edita</t>
         </is>
       </c>
       <c r="C97" s="14" t="n">
@@ -12883,7 +12883,7 @@
       </c>
       <c r="D97" s="14" t="inlineStr">
         <is>
-          <t>CT-01.01-07</t>
+          <t>complementar (sem CT na matriz)</t>
         </is>
       </c>
       <c r="E97" s="14" t="inlineStr">
@@ -12892,7 +12892,7 @@
         </is>
       </c>
       <c r="F97" s="14" t="n">
-        <v>0.6</v>
+        <v>2.849</v>
       </c>
       <c r="G97" s="14" t="inlineStr">
         <is>
@@ -12900,7 +12900,7 @@
         </is>
       </c>
       <c r="H97" s="14" t="n">
-        <v>0.592</v>
+        <v>4.547</v>
       </c>
     </row>
     <row r="98">
@@ -12911,7 +12911,7 @@
       </c>
       <c r="B98" s="14" t="inlineStr">
         <is>
-          <t>test_ct_01_03_01_aluno_nasce_sem_senha_com_perfil_aluno</t>
+          <t>test_ct_01_01_01_docente_nasce_inativo_e_sem_senha</t>
         </is>
       </c>
       <c r="C98" s="14" t="n">
@@ -12919,7 +12919,7 @@
       </c>
       <c r="D98" s="14" t="inlineStr">
         <is>
-          <t>CT-01.03-01</t>
+          <t>CT-01.01-01</t>
         </is>
       </c>
       <c r="E98" s="14" t="inlineStr">
@@ -12928,7 +12928,7 @@
         </is>
       </c>
       <c r="F98" s="14" t="n">
-        <v>0.579</v>
+        <v>0.806</v>
       </c>
       <c r="G98" s="14" t="inlineStr">
         <is>
@@ -12936,7 +12936,7 @@
         </is>
       </c>
       <c r="H98" s="14" t="n">
-        <v>0.584</v>
+        <v>1.54</v>
       </c>
     </row>
     <row r="99">
@@ -12947,7 +12947,7 @@
       </c>
       <c r="B99" s="14" t="inlineStr">
         <is>
-          <t>test_ct_01_03_03_indica_o_campo_duplicado</t>
+          <t>test_ct_01_01_02_campo_obrigatorio_vazio_responde_400</t>
         </is>
       </c>
       <c r="C99" s="14" t="n">
@@ -12955,7 +12955,7 @@
       </c>
       <c r="D99" s="14" t="inlineStr">
         <is>
-          <t>CT-01.03-03</t>
+          <t>CT-01.01-02</t>
         </is>
       </c>
       <c r="E99" s="14" t="inlineStr">
@@ -12964,7 +12964,7 @@
         </is>
       </c>
       <c r="F99" s="14" t="n">
-        <v>0.953</v>
+        <v>0.799</v>
       </c>
       <c r="G99" s="14" t="inlineStr">
         <is>
@@ -12972,7 +12972,7 @@
         </is>
       </c>
       <c r="H99" s="14" t="n">
-        <v>0.603</v>
+        <v>1.04</v>
       </c>
     </row>
     <row r="100">
@@ -12983,7 +12983,7 @@
       </c>
       <c r="B100" s="14" t="inlineStr">
         <is>
-          <t>test_ct_01_03_06_e_01_05_01_enfileira_ativacao_e_audita</t>
+          <t>test_ct_01_01_03_email_duplicado_ignora_maiusculas</t>
         </is>
       </c>
       <c r="C100" s="14" t="n">
@@ -12991,7 +12991,7 @@
       </c>
       <c r="D100" s="14" t="inlineStr">
         <is>
-          <t>CT-01.03-06, CT-01.05-01</t>
+          <t>CT-01.01-03</t>
         </is>
       </c>
       <c r="E100" s="14" t="inlineStr">
@@ -13000,7 +13000,7 @@
         </is>
       </c>
       <c r="F100" s="14" t="n">
-        <v>0.708</v>
+        <v>0.994</v>
       </c>
       <c r="G100" s="14" t="inlineStr">
         <is>
@@ -13008,7 +13008,7 @@
         </is>
       </c>
       <c r="H100" s="14" t="n">
-        <v>0.594</v>
+        <v>1.175</v>
       </c>
     </row>
     <row r="101">
@@ -13019,7 +13019,7 @@
       </c>
       <c r="B101" s="14" t="inlineStr">
         <is>
-          <t>test_ct_01_08_01_e_01_08_06_edicao_auditada_com_valor_anterior_e_novo</t>
+          <t>test_ct_01_01_05_coordenador_nao_exige_curso</t>
         </is>
       </c>
       <c r="C101" s="14" t="n">
@@ -13027,7 +13027,7 @@
       </c>
       <c r="D101" s="14" t="inlineStr">
         <is>
-          <t>CT-01.08-01, CT-01.08-06</t>
+          <t>CT-01.01-05</t>
         </is>
       </c>
       <c r="E101" s="14" t="inlineStr">
@@ -13036,7 +13036,7 @@
         </is>
       </c>
       <c r="F101" s="14" t="n">
-        <v>0.594</v>
+        <v>0.843</v>
       </c>
       <c r="G101" s="14" t="inlineStr">
         <is>
@@ -13044,7 +13044,7 @@
         </is>
       </c>
       <c r="H101" s="14" t="n">
-        <v>0.752</v>
+        <v>1.382</v>
       </c>
     </row>
     <row r="102">
@@ -13055,7 +13055,7 @@
       </c>
       <c r="B102" s="14" t="inlineStr">
         <is>
-          <t>test_ct_01_08_02_email_ou_matricula_de_outra_pessoa</t>
+          <t>test_ct_01_01_06_quem_nao_e_coordenador_recebe_403</t>
         </is>
       </c>
       <c r="C102" s="14" t="n">
@@ -13063,7 +13063,7 @@
       </c>
       <c r="D102" s="14" t="inlineStr">
         <is>
-          <t>CT-01.08-02</t>
+          <t>CT-01.01-06</t>
         </is>
       </c>
       <c r="E102" s="14" t="inlineStr">
@@ -13072,7 +13072,7 @@
         </is>
       </c>
       <c r="F102" s="14" t="n">
-        <v>0.735</v>
+        <v>1.102</v>
       </c>
       <c r="G102" s="14" t="inlineStr">
         <is>
@@ -13080,7 +13080,7 @@
         </is>
       </c>
       <c r="H102" s="14" t="n">
-        <v>0.768</v>
+        <v>1.96</v>
       </c>
     </row>
     <row r="103">
@@ -13091,7 +13091,7 @@
       </c>
       <c r="B103" s="14" t="inlineStr">
         <is>
-          <t>test_ct_01_08_03_e_01_08_04_inativado_nao_entra_e_reativado_volta</t>
+          <t>test_ct_01_01_07_criacao_fica_no_log</t>
         </is>
       </c>
       <c r="C103" s="14" t="n">
@@ -13099,7 +13099,7 @@
       </c>
       <c r="D103" s="14" t="inlineStr">
         <is>
-          <t>CT-01.06-08, CT-01.08-03, CT-01.08-04</t>
+          <t>CT-01.01-07</t>
         </is>
       </c>
       <c r="E103" s="14" t="inlineStr">
@@ -13108,7 +13108,7 @@
         </is>
       </c>
       <c r="F103" s="14" t="n">
-        <v>1.147</v>
+        <v>0.854</v>
       </c>
       <c r="G103" s="14" t="inlineStr">
         <is>
@@ -13116,7 +13116,7 @@
         </is>
       </c>
       <c r="H103" s="14" t="n">
-        <v>1.437</v>
+        <v>1.489</v>
       </c>
     </row>
     <row r="104">
@@ -13127,7 +13127,7 @@
       </c>
       <c r="B104" s="14" t="inlineStr">
         <is>
-          <t>test_hu0101_ca6_ninguem_altera_os_proprios_perfis</t>
+          <t>test_ct_01_03_01_aluno_nasce_sem_senha_com_perfil_aluno</t>
         </is>
       </c>
       <c r="C104" s="14" t="n">
@@ -13135,7 +13135,7 @@
       </c>
       <c r="D104" s="14" t="inlineStr">
         <is>
-          <t>complementar (sem CT na matriz)</t>
+          <t>CT-01.03-01</t>
         </is>
       </c>
       <c r="E104" s="14" t="inlineStr">
@@ -13144,7 +13144,7 @@
         </is>
       </c>
       <c r="F104" s="14" t="n">
-        <v>0.834</v>
+        <v>1.155</v>
       </c>
       <c r="G104" s="14" t="inlineStr">
         <is>
@@ -13152,7 +13152,7 @@
         </is>
       </c>
       <c r="H104" s="14" t="n">
-        <v>1.03</v>
+        <v>1.055</v>
       </c>
     </row>
     <row r="105">
@@ -13163,7 +13163,7 @@
       </c>
       <c r="B105" s="14" t="inlineStr">
         <is>
-          <t>test_hu0103_busca_e_filtro_por_curso</t>
+          <t>test_ct_01_03_03_indica_o_campo_duplicado</t>
         </is>
       </c>
       <c r="C105" s="14" t="n">
@@ -13171,7 +13171,7 @@
       </c>
       <c r="D105" s="14" t="inlineStr">
         <is>
-          <t>complementar (sem CT na matriz)</t>
+          <t>CT-01.03-03</t>
         </is>
       </c>
       <c r="E105" s="14" t="inlineStr">
@@ -13180,7 +13180,7 @@
         </is>
       </c>
       <c r="F105" s="14" t="n">
-        <v>1.099</v>
+        <v>0.878</v>
       </c>
       <c r="G105" s="14" t="inlineStr">
         <is>
@@ -13188,7 +13188,7 @@
         </is>
       </c>
       <c r="H105" s="14" t="n">
-        <v>1.022</v>
+        <v>1.447</v>
       </c>
     </row>
     <row r="106">
@@ -13199,7 +13199,7 @@
       </c>
       <c r="B106" s="14" t="inlineStr">
         <is>
-          <t>test_hu0103_e1_curso_fora_dos_contemplados</t>
+          <t>test_ct_01_03_06_e_01_05_01_enfileira_ativacao_e_audita</t>
         </is>
       </c>
       <c r="C106" s="14" t="n">
@@ -13207,7 +13207,7 @@
       </c>
       <c r="D106" s="14" t="inlineStr">
         <is>
-          <t>complementar (sem CT na matriz)</t>
+          <t>CT-01.03-06, CT-01.05-01</t>
         </is>
       </c>
       <c r="E106" s="14" t="inlineStr">
@@ -13216,7 +13216,7 @@
         </is>
       </c>
       <c r="F106" s="14" t="n">
-        <v>0.629</v>
+        <v>0.833</v>
       </c>
       <c r="G106" s="14" t="inlineStr">
         <is>
@@ -13224,7 +13224,7 @@
         </is>
       </c>
       <c r="H106" s="14" t="n">
-        <v>0.527</v>
+        <v>1.407</v>
       </c>
     </row>
     <row r="107">
@@ -13235,7 +13235,7 @@
       </c>
       <c r="B107" s="14" t="inlineStr">
         <is>
-          <t>test_hu0108_ca4_nao_existe_rota_de_exclusao</t>
+          <t>test_ct_01_08_01_e_01_08_06_edicao_auditada_com_valor_anterior_e_novo</t>
         </is>
       </c>
       <c r="C107" s="14" t="n">
@@ -13243,7 +13243,7 @@
       </c>
       <c r="D107" s="14" t="inlineStr">
         <is>
-          <t>complementar (sem CT na matriz)</t>
+          <t>CT-01.08-01, CT-01.08-06</t>
         </is>
       </c>
       <c r="E107" s="14" t="inlineStr">
@@ -13252,7 +13252,7 @@
         </is>
       </c>
       <c r="F107" s="14" t="n">
-        <v>0.76</v>
+        <v>0.923</v>
       </c>
       <c r="G107" s="14" t="inlineStr">
         <is>
@@ -13260,7 +13260,7 @@
         </is>
       </c>
       <c r="H107" s="14" t="n">
-        <v>0.698</v>
+        <v>1.17</v>
       </c>
     </row>
     <row r="108">
@@ -13271,7 +13271,7 @@
       </c>
       <c r="B108" s="14" t="inlineStr">
         <is>
-          <t>test_hu0108_coordenador_nao_inativa_a_si_mesmo</t>
+          <t>test_ct_01_08_02_email_ou_matricula_de_outra_pessoa</t>
         </is>
       </c>
       <c r="C108" s="14" t="n">
@@ -13279,29 +13279,245 @@
       </c>
       <c r="D108" s="14" t="inlineStr">
         <is>
+          <t>CT-01.08-02</t>
+        </is>
+      </c>
+      <c r="E108" s="14" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="F108" s="14" t="n">
+        <v>0.907</v>
+      </c>
+      <c r="G108" s="14" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H108" s="14" t="n">
+        <v>1.346</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="14" t="inlineStr">
+        <is>
+          <t>test_usuarios.py</t>
+        </is>
+      </c>
+      <c r="B109" s="14" t="inlineStr">
+        <is>
+          <t>test_ct_01_08_03_e_01_08_04_inativado_nao_entra_e_reativado_volta</t>
+        </is>
+      </c>
+      <c r="C109" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D109" s="14" t="inlineStr">
+        <is>
+          <t>CT-01.06-08, CT-01.08-03, CT-01.08-04</t>
+        </is>
+      </c>
+      <c r="E109" s="14" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="F109" s="14" t="n">
+        <v>1.389</v>
+      </c>
+      <c r="G109" s="14" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H109" s="14" t="n">
+        <v>2.326</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="14" t="inlineStr">
+        <is>
+          <t>test_usuarios.py</t>
+        </is>
+      </c>
+      <c r="B110" s="14" t="inlineStr">
+        <is>
+          <t>test_hu0101_ca6_ninguem_altera_os_proprios_perfis</t>
+        </is>
+      </c>
+      <c r="C110" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D110" s="14" t="inlineStr">
+        <is>
           <t>complementar (sem CT na matriz)</t>
         </is>
       </c>
-      <c r="E108" s="14" t="inlineStr">
-        <is>
-          <t>Aprovado</t>
-        </is>
-      </c>
-      <c r="F108" s="14" t="n">
-        <v>0.717</v>
-      </c>
-      <c r="G108" s="14" t="inlineStr">
-        <is>
-          <t>Aprovado</t>
-        </is>
-      </c>
-      <c r="H108" s="14" t="n">
-        <v>0.618</v>
+      <c r="E110" s="14" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="F110" s="14" t="n">
+        <v>1.012</v>
+      </c>
+      <c r="G110" s="14" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H110" s="14" t="n">
+        <v>2.056</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="14" t="inlineStr">
+        <is>
+          <t>test_usuarios.py</t>
+        </is>
+      </c>
+      <c r="B111" s="14" t="inlineStr">
+        <is>
+          <t>test_hu0103_busca_e_filtro_por_curso</t>
+        </is>
+      </c>
+      <c r="C111" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D111" s="14" t="inlineStr">
+        <is>
+          <t>complementar (sem CT na matriz)</t>
+        </is>
+      </c>
+      <c r="E111" s="14" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="F111" s="14" t="n">
+        <v>0.976</v>
+      </c>
+      <c r="G111" s="14" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H111" s="14" t="n">
+        <v>1.325</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="14" t="inlineStr">
+        <is>
+          <t>test_usuarios.py</t>
+        </is>
+      </c>
+      <c r="B112" s="14" t="inlineStr">
+        <is>
+          <t>test_hu0103_e1_curso_fora_dos_contemplados</t>
+        </is>
+      </c>
+      <c r="C112" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D112" s="14" t="inlineStr">
+        <is>
+          <t>complementar (sem CT na matriz)</t>
+        </is>
+      </c>
+      <c r="E112" s="14" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="F112" s="14" t="n">
+        <v>1.028</v>
+      </c>
+      <c r="G112" s="14" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H112" s="14" t="n">
+        <v>1.016</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="14" t="inlineStr">
+        <is>
+          <t>test_usuarios.py</t>
+        </is>
+      </c>
+      <c r="B113" s="14" t="inlineStr">
+        <is>
+          <t>test_hu0108_ca4_nao_existe_rota_de_exclusao</t>
+        </is>
+      </c>
+      <c r="C113" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D113" s="14" t="inlineStr">
+        <is>
+          <t>complementar (sem CT na matriz)</t>
+        </is>
+      </c>
+      <c r="E113" s="14" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="F113" s="14" t="n">
+        <v>0.823</v>
+      </c>
+      <c r="G113" s="14" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H113" s="14" t="n">
+        <v>1.386</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="14" t="inlineStr">
+        <is>
+          <t>test_usuarios.py</t>
+        </is>
+      </c>
+      <c r="B114" s="14" t="inlineStr">
+        <is>
+          <t>test_hu0108_coordenador_nao_inativa_a_si_mesmo</t>
+        </is>
+      </c>
+      <c r="C114" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D114" s="14" t="inlineStr">
+        <is>
+          <t>complementar (sem CT na matriz)</t>
+        </is>
+      </c>
+      <c r="E114" s="14" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="F114" s="14" t="n">
+        <v>0.8149999999999999</v>
+      </c>
+      <c r="G114" s="14" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H114" s="14" t="n">
+        <v>1.54</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H108"/>
-  <conditionalFormatting sqref="E2:E108">
+  <autoFilter ref="A1:H114"/>
+  <conditionalFormatting sqref="E2:E114">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$E2="Aprovado"</formula>
     </cfRule>
@@ -13318,7 +13534,7 @@
       <formula>$E2="Pulado"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G108">
+  <conditionalFormatting sqref="G2:G114">
     <cfRule type="expression" priority="6" dxfId="0">
       <formula>$G2="Aprovado"</formula>
     </cfRule>

</xml_diff>

<commit_message>
fix: confere o SHA-256 da foto na leitura (RNF06) e documenta o atendimento dos RNFs
- obter_foto recusa entregar arquivo alterado no banco, com teste
- arquitetura: seção 10 com RNF01 a RNF07 e divergências, linha de LGPD na segurança
- contrato da API: código 500 de arquivo que não confere
- suítes refeitas em SQLite e PostgreSQL (123 execuções, 0 falhas, 2 pulados)
</commit_message>
<xml_diff>
--- a/docs/testes/Relatorio_Execucao_Testes_SIGA_UEA.xlsx
+++ b/docs/testes/Relatorio_Execucao_Testes_SIGA_UEA.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Resumo" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Execucao por CT" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Testes automatizados" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Testes no navegador" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Desempenho RNF01" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Evidencias" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execucao por CT" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testes automatizados" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testes no navegador" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Desempenho RNF01" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidencias" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Execucao por CT'!$A$1:$O$103</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Testes automatizados'!$A$1:$H$114</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Testes automatizados'!$A$1:$H$115</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Testes no navegador'!$A$1:$F$60</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Evidencias'!$A$1:$B$29</definedName>
   </definedNames>
@@ -602,7 +602,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>20/10/2026 21:01 (America/Manaus)</t>
+          <t>20/10/2026 21:37 (America/Manaus)</t>
         </is>
       </c>
     </row>
@@ -614,7 +614,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>449f0e6 · branch dev · repositório SIGA-UEA/sigauea</t>
+          <t>838df67 · branch dev · repositório SIGA-UEA/sigauea</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B18" s="8">
-        <f>COUNTIF('Testes automatizados'!$E$2:$E$114,"Aprovado")</f>
+        <f>COUNTIF('Testes automatizados'!$E$2:$E$115,"Aprovado")</f>
         <v/>
       </c>
     </row>
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="B19" s="8">
-        <f>COUNTIF('Testes automatizados'!$E$2:$E$114,"Pulado")</f>
+        <f>COUNTIF('Testes automatizados'!$E$2:$E$115,"Pulado")</f>
         <v/>
       </c>
     </row>
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B20" s="8">
-        <f>COUNTIF('Testes automatizados'!$E$2:$E$114,"Reprovado")</f>
+        <f>COUNTIF('Testes automatizados'!$E$2:$E$115,"Reprovado")</f>
         <v/>
       </c>
     </row>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B21" s="8">
-        <f>COUNTIF('Testes automatizados'!$G$2:$G$114,"Aprovado")</f>
+        <f>COUNTIF('Testes automatizados'!$G$2:$G$115,"Aprovado")</f>
         <v/>
       </c>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="B22" s="8">
-        <f>COUNTIF('Testes automatizados'!$G$2:$G$114,"Pulado")</f>
+        <f>COUNTIF('Testes automatizados'!$G$2:$G$115,"Pulado")</f>
         <v/>
       </c>
     </row>
@@ -801,7 +801,7 @@
         </is>
       </c>
       <c r="B23" s="8">
-        <f>COUNTIF('Testes automatizados'!$G$2:$G$114,"Reprovado")</f>
+        <f>COUNTIF('Testes automatizados'!$G$2:$G$115,"Reprovado")</f>
         <v/>
       </c>
     </row>
@@ -852,7 +852,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Funções de teste da API: 113 (122 execuções contando os parâmetros). Um teste pulado é um caso Pendente na matriz: a funcionalidade ainda não existe (CT-01.10-06 depende do módulo de ideias; CT-06.01-04, da troca de orientador pela coordenação).</t>
+          <t>Funções de teste da API: 114 (123 execuções contando os parâmetros). Um teste pulado é um caso Pendente na matriz: a funcionalidade ainda não existe (CT-01.10-06 depende do módulo de ideias; CT-06.01-04, da troca de orientador pela coordenação).</t>
         </is>
       </c>
     </row>
@@ -9392,7 +9392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H114"/>
+  <dimension ref="A1:H115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -9472,7 +9472,7 @@
         </is>
       </c>
       <c r="F2" s="14" t="n">
-        <v>1.128</v>
+        <v>1.094</v>
       </c>
       <c r="G2" s="14" t="inlineStr">
         <is>
@@ -9480,7 +9480,7 @@
         </is>
       </c>
       <c r="H2" s="14" t="n">
-        <v>0.966</v>
+        <v>1.005</v>
       </c>
     </row>
     <row r="3">
@@ -9508,7 +9508,7 @@
         </is>
       </c>
       <c r="F3" s="14" t="n">
-        <v>4.388</v>
+        <v>4.484</v>
       </c>
       <c r="G3" s="14" t="inlineStr">
         <is>
@@ -9516,7 +9516,7 @@
         </is>
       </c>
       <c r="H3" s="14" t="n">
-        <v>3.963</v>
+        <v>3.798</v>
       </c>
     </row>
     <row r="4">
@@ -9544,7 +9544,7 @@
         </is>
       </c>
       <c r="F4" s="14" t="n">
-        <v>0.889</v>
+        <v>0.913</v>
       </c>
       <c r="G4" s="14" t="inlineStr">
         <is>
@@ -9552,7 +9552,7 @@
         </is>
       </c>
       <c r="H4" s="14" t="n">
-        <v>0.849</v>
+        <v>0.802</v>
       </c>
     </row>
     <row r="5">
@@ -9580,7 +9580,7 @@
         </is>
       </c>
       <c r="F5" s="14" t="n">
-        <v>1.016</v>
+        <v>1.173</v>
       </c>
       <c r="G5" s="14" t="inlineStr">
         <is>
@@ -9588,7 +9588,7 @@
         </is>
       </c>
       <c r="H5" s="14" t="n">
-        <v>0.9330000000000001</v>
+        <v>1.025</v>
       </c>
     </row>
     <row r="6">
@@ -9616,7 +9616,7 @@
         </is>
       </c>
       <c r="F6" s="14" t="n">
-        <v>1.106</v>
+        <v>0.835</v>
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
@@ -9624,7 +9624,7 @@
         </is>
       </c>
       <c r="H6" s="14" t="n">
-        <v>0.748</v>
+        <v>0.705</v>
       </c>
     </row>
     <row r="7">
@@ -9652,7 +9652,7 @@
         </is>
       </c>
       <c r="F7" s="14" t="n">
-        <v>0.944</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
@@ -9660,7 +9660,7 @@
         </is>
       </c>
       <c r="H7" s="14" t="n">
-        <v>0.871</v>
+        <v>0.9330000000000001</v>
       </c>
     </row>
     <row r="8">
@@ -9688,7 +9688,7 @@
         </is>
       </c>
       <c r="F8" s="14" t="n">
-        <v>0.946</v>
+        <v>1.124</v>
       </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
@@ -9696,7 +9696,7 @@
         </is>
       </c>
       <c r="H8" s="14" t="n">
-        <v>0.829</v>
+        <v>0.868</v>
       </c>
     </row>
     <row r="9">
@@ -9724,7 +9724,7 @@
         </is>
       </c>
       <c r="F9" s="14" t="n">
-        <v>0.71</v>
+        <v>0.8</v>
       </c>
       <c r="G9" s="14" t="inlineStr">
         <is>
@@ -9732,7 +9732,7 @@
         </is>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.709</v>
+        <v>0.869</v>
       </c>
     </row>
     <row r="10">
@@ -9760,7 +9760,7 @@
         </is>
       </c>
       <c r="F10" s="14" t="n">
-        <v>0.781</v>
+        <v>0.908</v>
       </c>
       <c r="G10" s="14" t="inlineStr">
         <is>
@@ -9768,7 +9768,7 @@
         </is>
       </c>
       <c r="H10" s="14" t="n">
-        <v>0.794</v>
+        <v>0.758</v>
       </c>
     </row>
     <row r="11">
@@ -9796,7 +9796,7 @@
         </is>
       </c>
       <c r="F11" s="14" t="n">
-        <v>0.986</v>
+        <v>1.168</v>
       </c>
       <c r="G11" s="14" t="inlineStr">
         <is>
@@ -9804,7 +9804,7 @@
         </is>
       </c>
       <c r="H11" s="14" t="n">
-        <v>1.033</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="12">
@@ -9832,7 +9832,7 @@
         </is>
       </c>
       <c r="F12" s="14" t="n">
-        <v>0.764</v>
+        <v>1.021</v>
       </c>
       <c r="G12" s="14" t="inlineStr">
         <is>
@@ -9840,7 +9840,7 @@
         </is>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.736</v>
+        <v>0.706</v>
       </c>
     </row>
     <row r="13">
@@ -9868,7 +9868,7 @@
         </is>
       </c>
       <c r="F13" s="14" t="n">
-        <v>0.6879999999999999</v>
+        <v>0.6909999999999999</v>
       </c>
       <c r="G13" s="14" t="inlineStr">
         <is>
@@ -9876,7 +9876,7 @@
         </is>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.618</v>
+        <v>0.59</v>
       </c>
     </row>
     <row r="14">
@@ -9904,7 +9904,7 @@
         </is>
       </c>
       <c r="F14" s="14" t="n">
-        <v>1.589</v>
+        <v>1.513</v>
       </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
@@ -9912,7 +9912,7 @@
         </is>
       </c>
       <c r="H14" s="14" t="n">
-        <v>1.218</v>
+        <v>1.291</v>
       </c>
     </row>
     <row r="15">
@@ -9940,7 +9940,7 @@
         </is>
       </c>
       <c r="F15" s="14" t="n">
-        <v>0.719</v>
+        <v>0.655</v>
       </c>
       <c r="G15" s="14" t="inlineStr">
         <is>
@@ -9948,7 +9948,7 @@
         </is>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.875</v>
+        <v>0.646</v>
       </c>
     </row>
     <row r="16">
@@ -9976,7 +9976,7 @@
         </is>
       </c>
       <c r="F16" s="14" t="n">
-        <v>0.729</v>
+        <v>0.843</v>
       </c>
       <c r="G16" s="14" t="inlineStr">
         <is>
@@ -9984,7 +9984,7 @@
         </is>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.623</v>
+        <v>0.697</v>
       </c>
     </row>
     <row r="17">
@@ -10012,7 +10012,7 @@
         </is>
       </c>
       <c r="F17" s="14" t="n">
-        <v>0.752</v>
+        <v>0.8080000000000001</v>
       </c>
       <c r="G17" s="14" t="inlineStr">
         <is>
@@ -10020,7 +10020,7 @@
         </is>
       </c>
       <c r="H17" s="14" t="n">
-        <v>0.994</v>
+        <v>0.758</v>
       </c>
     </row>
     <row r="18">
@@ -10048,7 +10048,7 @@
         </is>
       </c>
       <c r="F18" s="14" t="n">
-        <v>0.974</v>
+        <v>1.017</v>
       </c>
       <c r="G18" s="14" t="inlineStr">
         <is>
@@ -10056,7 +10056,7 @@
         </is>
       </c>
       <c r="H18" s="14" t="n">
-        <v>0.82</v>
+        <v>0.854</v>
       </c>
     </row>
     <row r="19">
@@ -10084,7 +10084,7 @@
         </is>
       </c>
       <c r="F19" s="14" t="n">
-        <v>1.27</v>
+        <v>1.022</v>
       </c>
       <c r="G19" s="14" t="inlineStr">
         <is>
@@ -10092,7 +10092,7 @@
         </is>
       </c>
       <c r="H19" s="14" t="n">
-        <v>0.86</v>
+        <v>0.962</v>
       </c>
     </row>
     <row r="20">
@@ -10120,7 +10120,7 @@
         </is>
       </c>
       <c r="F20" s="14" t="n">
-        <v>0.856</v>
+        <v>0.847</v>
       </c>
       <c r="G20" s="14" t="inlineStr">
         <is>
@@ -10128,7 +10128,7 @@
         </is>
       </c>
       <c r="H20" s="14" t="n">
-        <v>0.743</v>
+        <v>0.776</v>
       </c>
     </row>
     <row r="21">
@@ -10156,7 +10156,7 @@
         </is>
       </c>
       <c r="F21" s="14" t="n">
-        <v>2.576</v>
+        <v>2.521</v>
       </c>
       <c r="G21" s="14" t="inlineStr">
         <is>
@@ -10164,7 +10164,7 @@
         </is>
       </c>
       <c r="H21" s="14" t="n">
-        <v>2.397</v>
+        <v>2.291</v>
       </c>
     </row>
     <row r="22">
@@ -10192,7 +10192,7 @@
         </is>
       </c>
       <c r="F22" s="14" t="n">
-        <v>1.171</v>
+        <v>0.882</v>
       </c>
       <c r="G22" s="14" t="inlineStr">
         <is>
@@ -10200,7 +10200,7 @@
         </is>
       </c>
       <c r="H22" s="14" t="n">
-        <v>0.896</v>
+        <v>0.771</v>
       </c>
     </row>
     <row r="23">
@@ -10228,7 +10228,7 @@
         </is>
       </c>
       <c r="F23" s="14" t="n">
-        <v>0.741</v>
+        <v>0.831</v>
       </c>
       <c r="G23" s="14" t="inlineStr">
         <is>
@@ -10236,7 +10236,7 @@
         </is>
       </c>
       <c r="H23" s="14" t="n">
-        <v>0.869</v>
+        <v>0.659</v>
       </c>
     </row>
     <row r="24">
@@ -10264,7 +10264,7 @@
         </is>
       </c>
       <c r="F24" s="14" t="n">
-        <v>0.783</v>
+        <v>1.097</v>
       </c>
       <c r="G24" s="14" t="inlineStr">
         <is>
@@ -10272,7 +10272,7 @@
         </is>
       </c>
       <c r="H24" s="14" t="n">
-        <v>0.793</v>
+        <v>0.804</v>
       </c>
     </row>
     <row r="25">
@@ -10300,7 +10300,7 @@
         </is>
       </c>
       <c r="F25" s="14" t="n">
-        <v>0.79</v>
+        <v>0.819</v>
       </c>
       <c r="G25" s="14" t="inlineStr">
         <is>
@@ -10308,7 +10308,7 @@
         </is>
       </c>
       <c r="H25" s="14" t="n">
-        <v>0.839</v>
+        <v>0.644</v>
       </c>
     </row>
     <row r="26">
@@ -10336,7 +10336,7 @@
         </is>
       </c>
       <c r="F26" s="14" t="n">
-        <v>1.04</v>
+        <v>1.074</v>
       </c>
       <c r="G26" s="14" t="inlineStr">
         <is>
@@ -10344,7 +10344,7 @@
         </is>
       </c>
       <c r="H26" s="14" t="n">
-        <v>1.13</v>
+        <v>0.988</v>
       </c>
     </row>
     <row r="27">
@@ -10372,7 +10372,7 @@
         </is>
       </c>
       <c r="F27" s="14" t="n">
-        <v>0.571</v>
+        <v>0.664</v>
       </c>
       <c r="G27" s="14" t="inlineStr">
         <is>
@@ -10380,7 +10380,7 @@
         </is>
       </c>
       <c r="H27" s="14" t="n">
-        <v>0.53</v>
+        <v>0.656</v>
       </c>
     </row>
     <row r="28">
@@ -10408,7 +10408,7 @@
         </is>
       </c>
       <c r="F28" s="14" t="n">
-        <v>1.572</v>
+        <v>1.265</v>
       </c>
       <c r="G28" s="14" t="inlineStr">
         <is>
@@ -10416,7 +10416,7 @@
         </is>
       </c>
       <c r="H28" s="14" t="n">
-        <v>1.085</v>
+        <v>1.089</v>
       </c>
     </row>
     <row r="29">
@@ -10480,7 +10480,7 @@
         </is>
       </c>
       <c r="F30" s="14" t="n">
-        <v>2.603</v>
+        <v>2.381</v>
       </c>
       <c r="G30" s="14" t="inlineStr">
         <is>
@@ -10488,7 +10488,7 @@
         </is>
       </c>
       <c r="H30" s="14" t="n">
-        <v>2.11</v>
+        <v>2.016</v>
       </c>
     </row>
     <row r="31">
@@ -10516,7 +10516,7 @@
         </is>
       </c>
       <c r="F31" s="14" t="n">
-        <v>2.092</v>
+        <v>1.911</v>
       </c>
       <c r="G31" s="14" t="inlineStr">
         <is>
@@ -10524,7 +10524,7 @@
         </is>
       </c>
       <c r="H31" s="14" t="n">
-        <v>1.795</v>
+        <v>1.614</v>
       </c>
     </row>
     <row r="32">
@@ -10552,7 +10552,7 @@
         </is>
       </c>
       <c r="F32" s="14" t="n">
-        <v>1.94</v>
+        <v>1.931</v>
       </c>
       <c r="G32" s="14" t="inlineStr">
         <is>
@@ -10560,7 +10560,7 @@
         </is>
       </c>
       <c r="H32" s="14" t="n">
-        <v>1.782</v>
+        <v>1.746</v>
       </c>
     </row>
     <row r="33">
@@ -10588,7 +10588,7 @@
         </is>
       </c>
       <c r="F33" s="14" t="n">
-        <v>2.929</v>
+        <v>2.491</v>
       </c>
       <c r="G33" s="14" t="inlineStr">
         <is>
@@ -10596,7 +10596,7 @@
         </is>
       </c>
       <c r="H33" s="14" t="n">
-        <v>2.108</v>
+        <v>2.055</v>
       </c>
     </row>
     <row r="34">
@@ -10624,7 +10624,7 @@
         </is>
       </c>
       <c r="F34" s="14" t="n">
-        <v>6.11</v>
+        <v>6.284</v>
       </c>
       <c r="G34" s="14" t="inlineStr">
         <is>
@@ -10632,7 +10632,7 @@
         </is>
       </c>
       <c r="H34" s="14" t="n">
-        <v>4.898</v>
+        <v>4.541</v>
       </c>
     </row>
     <row r="35">
@@ -10660,7 +10660,7 @@
         </is>
       </c>
       <c r="F35" s="14" t="n">
-        <v>1.875</v>
+        <v>2.091</v>
       </c>
       <c r="G35" s="14" t="inlineStr">
         <is>
@@ -10668,7 +10668,7 @@
         </is>
       </c>
       <c r="H35" s="14" t="n">
-        <v>1.75</v>
+        <v>1.791</v>
       </c>
     </row>
     <row r="36">
@@ -10696,7 +10696,7 @@
         </is>
       </c>
       <c r="F36" s="14" t="n">
-        <v>2.107</v>
+        <v>2.041</v>
       </c>
       <c r="G36" s="14" t="inlineStr">
         <is>
@@ -10704,7 +10704,7 @@
         </is>
       </c>
       <c r="H36" s="14" t="n">
-        <v>1.918</v>
+        <v>1.798</v>
       </c>
     </row>
     <row r="37">
@@ -10768,7 +10768,7 @@
         </is>
       </c>
       <c r="F38" s="14" t="n">
-        <v>3.466</v>
+        <v>2.74</v>
       </c>
       <c r="G38" s="14" t="inlineStr">
         <is>
@@ -10776,7 +10776,7 @@
         </is>
       </c>
       <c r="H38" s="14" t="n">
-        <v>2.416</v>
+        <v>2.088</v>
       </c>
     </row>
     <row r="39">
@@ -10804,7 +10804,7 @@
         </is>
       </c>
       <c r="F39" s="14" t="n">
-        <v>2.638</v>
+        <v>2.282</v>
       </c>
       <c r="G39" s="14" t="inlineStr">
         <is>
@@ -10812,7 +10812,7 @@
         </is>
       </c>
       <c r="H39" s="14" t="n">
-        <v>2.022</v>
+        <v>1.844</v>
       </c>
     </row>
     <row r="40">
@@ -10840,7 +10840,7 @@
         </is>
       </c>
       <c r="F40" s="14" t="n">
-        <v>1.086</v>
+        <v>0.9370000000000001</v>
       </c>
       <c r="G40" s="14" t="inlineStr">
         <is>
@@ -10848,7 +10848,7 @@
         </is>
       </c>
       <c r="H40" s="14" t="n">
-        <v>0.804</v>
+        <v>0.8159999999999999</v>
       </c>
     </row>
     <row r="41">
@@ -10876,7 +10876,7 @@
         </is>
       </c>
       <c r="F41" s="14" t="n">
-        <v>1.683</v>
+        <v>1.214</v>
       </c>
       <c r="G41" s="14" t="inlineStr">
         <is>
@@ -10884,7 +10884,7 @@
         </is>
       </c>
       <c r="H41" s="14" t="n">
-        <v>1.201</v>
+        <v>1.214</v>
       </c>
     </row>
     <row r="42">
@@ -10912,7 +10912,7 @@
         </is>
       </c>
       <c r="F42" s="14" t="n">
-        <v>1.425</v>
+        <v>1.648</v>
       </c>
       <c r="G42" s="14" t="inlineStr">
         <is>
@@ -10920,7 +10920,7 @@
         </is>
       </c>
       <c r="H42" s="14" t="n">
-        <v>1.388</v>
+        <v>1.119</v>
       </c>
     </row>
     <row r="43">
@@ -10948,7 +10948,7 @@
         </is>
       </c>
       <c r="F43" s="14" t="n">
-        <v>1.329</v>
+        <v>1.261</v>
       </c>
       <c r="G43" s="14" t="inlineStr">
         <is>
@@ -10956,7 +10956,7 @@
         </is>
       </c>
       <c r="H43" s="14" t="n">
-        <v>1.047</v>
+        <v>1.145</v>
       </c>
     </row>
     <row r="44">
@@ -10984,7 +10984,7 @@
         </is>
       </c>
       <c r="F44" s="14" t="n">
-        <v>1.31</v>
+        <v>1.184</v>
       </c>
       <c r="G44" s="14" t="inlineStr">
         <is>
@@ -10992,7 +10992,7 @@
         </is>
       </c>
       <c r="H44" s="14" t="n">
-        <v>1.226</v>
+        <v>1.294</v>
       </c>
     </row>
     <row r="45">
@@ -11020,7 +11020,7 @@
         </is>
       </c>
       <c r="F45" s="14" t="n">
-        <v>1.69</v>
+        <v>1.2</v>
       </c>
       <c r="G45" s="14" t="inlineStr">
         <is>
@@ -11028,7 +11028,7 @@
         </is>
       </c>
       <c r="H45" s="14" t="n">
-        <v>1.327</v>
+        <v>1.175</v>
       </c>
     </row>
     <row r="46">
@@ -11056,7 +11056,7 @@
         </is>
       </c>
       <c r="F46" s="14" t="n">
-        <v>1.807</v>
+        <v>1.578</v>
       </c>
       <c r="G46" s="14" t="inlineStr">
         <is>
@@ -11064,7 +11064,7 @@
         </is>
       </c>
       <c r="H46" s="14" t="n">
-        <v>1.736</v>
+        <v>1.359</v>
       </c>
     </row>
     <row r="47">
@@ -11092,7 +11092,7 @@
         </is>
       </c>
       <c r="F47" s="14" t="n">
-        <v>1.114</v>
+        <v>0.848</v>
       </c>
       <c r="G47" s="14" t="inlineStr">
         <is>
@@ -11100,7 +11100,7 @@
         </is>
       </c>
       <c r="H47" s="14" t="n">
-        <v>0.984</v>
+        <v>0.849</v>
       </c>
     </row>
     <row r="48">
@@ -11128,7 +11128,7 @@
         </is>
       </c>
       <c r="F48" s="14" t="n">
-        <v>0.952</v>
+        <v>0.784</v>
       </c>
       <c r="G48" s="14" t="inlineStr">
         <is>
@@ -11136,7 +11136,7 @@
         </is>
       </c>
       <c r="H48" s="14" t="n">
-        <v>0.766</v>
+        <v>0.733</v>
       </c>
     </row>
     <row r="49">
@@ -11164,7 +11164,7 @@
         </is>
       </c>
       <c r="F49" s="14" t="n">
-        <v>1.146</v>
+        <v>0.9389999999999999</v>
       </c>
       <c r="G49" s="14" t="inlineStr">
         <is>
@@ -11172,7 +11172,7 @@
         </is>
       </c>
       <c r="H49" s="14" t="n">
-        <v>0.885</v>
+        <v>1.068</v>
       </c>
     </row>
     <row r="50">
@@ -11200,7 +11200,7 @@
         </is>
       </c>
       <c r="F50" s="14" t="n">
-        <v>1.424</v>
+        <v>1.151</v>
       </c>
       <c r="G50" s="14" t="inlineStr">
         <is>
@@ -11208,7 +11208,7 @@
         </is>
       </c>
       <c r="H50" s="14" t="n">
-        <v>1.055</v>
+        <v>1.081</v>
       </c>
     </row>
     <row r="51">
@@ -11236,7 +11236,7 @@
         </is>
       </c>
       <c r="F51" s="14" t="n">
-        <v>1.717</v>
+        <v>1.211</v>
       </c>
       <c r="G51" s="14" t="inlineStr">
         <is>
@@ -11244,7 +11244,7 @@
         </is>
       </c>
       <c r="H51" s="14" t="n">
-        <v>1.226</v>
+        <v>1.296</v>
       </c>
     </row>
     <row r="52">
@@ -11272,7 +11272,7 @@
         </is>
       </c>
       <c r="F52" s="14" t="n">
-        <v>1.631</v>
+        <v>1.573</v>
       </c>
       <c r="G52" s="14" t="inlineStr">
         <is>
@@ -11280,7 +11280,7 @@
         </is>
       </c>
       <c r="H52" s="14" t="n">
-        <v>1.071</v>
+        <v>1.18</v>
       </c>
     </row>
     <row r="53">
@@ -11308,7 +11308,7 @@
         </is>
       </c>
       <c r="F53" s="14" t="n">
-        <v>1.375</v>
+        <v>1.183</v>
       </c>
       <c r="G53" s="14" t="inlineStr">
         <is>
@@ -11316,7 +11316,7 @@
         </is>
       </c>
       <c r="H53" s="14" t="n">
-        <v>0.9379999999999999</v>
+        <v>1.009</v>
       </c>
     </row>
     <row r="54">
@@ -11344,7 +11344,7 @@
         </is>
       </c>
       <c r="F54" s="14" t="n">
-        <v>1.451</v>
+        <v>1.102</v>
       </c>
       <c r="G54" s="14" t="inlineStr">
         <is>
@@ -11352,7 +11352,7 @@
         </is>
       </c>
       <c r="H54" s="14" t="n">
-        <v>1.003</v>
+        <v>1.033</v>
       </c>
     </row>
     <row r="55">
@@ -11380,7 +11380,7 @@
         </is>
       </c>
       <c r="F55" s="14" t="n">
-        <v>1.436</v>
+        <v>1.062</v>
       </c>
       <c r="G55" s="14" t="inlineStr">
         <is>
@@ -11388,7 +11388,7 @@
         </is>
       </c>
       <c r="H55" s="14" t="n">
-        <v>0.983</v>
+        <v>0.928</v>
       </c>
     </row>
     <row r="56">
@@ -11416,7 +11416,7 @@
         </is>
       </c>
       <c r="F56" s="14" t="n">
-        <v>1.481</v>
+        <v>1.241</v>
       </c>
       <c r="G56" s="14" t="inlineStr">
         <is>
@@ -11424,7 +11424,7 @@
         </is>
       </c>
       <c r="H56" s="14" t="n">
-        <v>1.156</v>
+        <v>1.06</v>
       </c>
     </row>
     <row r="57">
@@ -11452,7 +11452,7 @@
         </is>
       </c>
       <c r="F57" s="14" t="n">
-        <v>1.426</v>
+        <v>1.368</v>
       </c>
       <c r="G57" s="14" t="inlineStr">
         <is>
@@ -11460,7 +11460,7 @@
         </is>
       </c>
       <c r="H57" s="14" t="n">
-        <v>1.098</v>
+        <v>1.103</v>
       </c>
     </row>
     <row r="58">
@@ -11488,7 +11488,7 @@
         </is>
       </c>
       <c r="F58" s="14" t="n">
-        <v>1.401</v>
+        <v>1.057</v>
       </c>
       <c r="G58" s="14" t="inlineStr">
         <is>
@@ -11496,7 +11496,7 @@
         </is>
       </c>
       <c r="H58" s="14" t="n">
-        <v>1.332</v>
+        <v>0.998</v>
       </c>
     </row>
     <row r="59">
@@ -11524,7 +11524,7 @@
         </is>
       </c>
       <c r="F59" s="14" t="n">
-        <v>1.429</v>
+        <v>1.077</v>
       </c>
       <c r="G59" s="14" t="inlineStr">
         <is>
@@ -11532,7 +11532,7 @@
         </is>
       </c>
       <c r="H59" s="14" t="n">
-        <v>1.33</v>
+        <v>1.033</v>
       </c>
     </row>
     <row r="60">
@@ -11560,7 +11560,7 @@
         </is>
       </c>
       <c r="F60" s="14" t="n">
-        <v>1.386</v>
+        <v>1.108</v>
       </c>
       <c r="G60" s="14" t="inlineStr">
         <is>
@@ -11568,7 +11568,7 @@
         </is>
       </c>
       <c r="H60" s="14" t="n">
-        <v>1.05</v>
+        <v>0.953</v>
       </c>
     </row>
     <row r="61">
@@ -11596,7 +11596,7 @@
         </is>
       </c>
       <c r="F61" s="14" t="n">
-        <v>1.221</v>
+        <v>0.891</v>
       </c>
       <c r="G61" s="14" t="inlineStr">
         <is>
@@ -11604,7 +11604,7 @@
         </is>
       </c>
       <c r="H61" s="14" t="n">
-        <v>0.844</v>
+        <v>0.727</v>
       </c>
     </row>
     <row r="62">
@@ -11632,7 +11632,7 @@
         </is>
       </c>
       <c r="F62" s="14" t="n">
-        <v>1.537</v>
+        <v>1.107</v>
       </c>
       <c r="G62" s="14" t="inlineStr">
         <is>
@@ -11640,7 +11640,7 @@
         </is>
       </c>
       <c r="H62" s="14" t="n">
-        <v>1.044</v>
+        <v>1.067</v>
       </c>
     </row>
     <row r="63">
@@ -11668,7 +11668,7 @@
         </is>
       </c>
       <c r="F63" s="14" t="n">
-        <v>2.498</v>
+        <v>1.986</v>
       </c>
       <c r="G63" s="14" t="inlineStr">
         <is>
@@ -11676,7 +11676,7 @@
         </is>
       </c>
       <c r="H63" s="14" t="n">
-        <v>1.612</v>
+        <v>1.657</v>
       </c>
     </row>
     <row r="64">
@@ -11704,7 +11704,7 @@
         </is>
       </c>
       <c r="F64" s="14" t="n">
-        <v>1.153</v>
+        <v>0.8169999999999999</v>
       </c>
       <c r="G64" s="14" t="inlineStr">
         <is>
@@ -11712,7 +11712,7 @@
         </is>
       </c>
       <c r="H64" s="14" t="n">
-        <v>0.739</v>
+        <v>0.865</v>
       </c>
     </row>
     <row r="65">
@@ -11740,7 +11740,7 @@
         </is>
       </c>
       <c r="F65" s="14" t="n">
-        <v>0.977</v>
+        <v>0.8080000000000001</v>
       </c>
       <c r="G65" s="14" t="inlineStr">
         <is>
@@ -11748,7 +11748,7 @@
         </is>
       </c>
       <c r="H65" s="14" t="n">
-        <v>0.716</v>
+        <v>0.995</v>
       </c>
     </row>
     <row r="66">
@@ -11776,7 +11776,7 @@
         </is>
       </c>
       <c r="F66" s="14" t="n">
-        <v>1.109</v>
+        <v>0.85</v>
       </c>
       <c r="G66" s="14" t="inlineStr">
         <is>
@@ -11784,7 +11784,7 @@
         </is>
       </c>
       <c r="H66" s="14" t="n">
-        <v>1.947</v>
+        <v>0.892</v>
       </c>
     </row>
     <row r="67">
@@ -11812,7 +11812,7 @@
         </is>
       </c>
       <c r="F67" s="14" t="n">
-        <v>0.72</v>
+        <v>0.643</v>
       </c>
       <c r="G67" s="14" t="inlineStr">
         <is>
@@ -11820,7 +11820,7 @@
         </is>
       </c>
       <c r="H67" s="14" t="n">
-        <v>0.582</v>
+        <v>0.425</v>
       </c>
     </row>
     <row r="68">
@@ -11848,7 +11848,7 @@
         </is>
       </c>
       <c r="F68" s="14" t="n">
-        <v>2.828</v>
+        <v>1.847</v>
       </c>
       <c r="G68" s="14" t="inlineStr">
         <is>
@@ -11856,7 +11856,7 @@
         </is>
       </c>
       <c r="H68" s="14" t="n">
-        <v>1.744</v>
+        <v>1.985</v>
       </c>
     </row>
     <row r="69">
@@ -11884,7 +11884,7 @@
         </is>
       </c>
       <c r="F69" s="14" t="n">
-        <v>2.898</v>
+        <v>2.083</v>
       </c>
       <c r="G69" s="14" t="inlineStr">
         <is>
@@ -11892,7 +11892,7 @@
         </is>
       </c>
       <c r="H69" s="14" t="n">
-        <v>2.131</v>
+        <v>2.266</v>
       </c>
     </row>
     <row r="70">
@@ -11903,7 +11903,7 @@
       </c>
       <c r="B70" s="14" t="inlineStr">
         <is>
-          <t>test_so_a_coordenacao_remove_foto_de_outra_pessoa</t>
+          <t>test_rnf06_foto_alterada_no_banco_nao_e_entregue</t>
         </is>
       </c>
       <c r="C70" s="14" t="n">
@@ -11920,7 +11920,7 @@
         </is>
       </c>
       <c r="F70" s="14" t="n">
-        <v>2.754</v>
+        <v>0.976</v>
       </c>
       <c r="G70" s="14" t="inlineStr">
         <is>
@@ -11928,18 +11928,18 @@
         </is>
       </c>
       <c r="H70" s="14" t="n">
-        <v>3.522</v>
+        <v>0.745</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="14" t="inlineStr">
         <is>
-          <t>test_tcc.py</t>
+          <t>test_rotas_restantes.py</t>
         </is>
       </c>
       <c r="B71" s="14" t="inlineStr">
         <is>
-          <t>test_ct_01_03_04_aluno_de_outro_curso_entra_e_mantem_o_curso</t>
+          <t>test_so_a_coordenacao_remove_foto_de_outra_pessoa</t>
         </is>
       </c>
       <c r="C71" s="14" t="n">
@@ -11947,7 +11947,7 @@
       </c>
       <c r="D71" s="14" t="inlineStr">
         <is>
-          <t>CT-01.03-04</t>
+          <t>complementar (sem CT na matriz)</t>
         </is>
       </c>
       <c r="E71" s="14" t="inlineStr">
@@ -11956,7 +11956,7 @@
         </is>
       </c>
       <c r="F71" s="14" t="n">
-        <v>2.631</v>
+        <v>1.886</v>
       </c>
       <c r="G71" s="14" t="inlineStr">
         <is>
@@ -11964,7 +11964,7 @@
         </is>
       </c>
       <c r="H71" s="14" t="n">
-        <v>3.42</v>
+        <v>1.798</v>
       </c>
     </row>
     <row r="72">
@@ -11975,7 +11975,7 @@
       </c>
       <c r="B72" s="14" t="inlineStr">
         <is>
-          <t>test_ct_03_01_01_formulario_traz_turma_orientadores_e_areas</t>
+          <t>test_ct_01_03_04_aluno_de_outro_curso_entra_e_mantem_o_curso</t>
         </is>
       </c>
       <c r="C72" s="14" t="n">
@@ -11983,7 +11983,7 @@
       </c>
       <c r="D72" s="14" t="inlineStr">
         <is>
-          <t>CT-03.01-01</t>
+          <t>CT-01.03-04</t>
         </is>
       </c>
       <c r="E72" s="14" t="inlineStr">
@@ -11992,7 +11992,7 @@
         </is>
       </c>
       <c r="F72" s="14" t="n">
-        <v>2.094</v>
+        <v>1.945</v>
       </c>
       <c r="G72" s="14" t="inlineStr">
         <is>
@@ -12000,7 +12000,7 @@
         </is>
       </c>
       <c r="H72" s="14" t="n">
-        <v>2.017</v>
+        <v>1.969</v>
       </c>
     </row>
     <row r="73">
@@ -12011,7 +12011,7 @@
       </c>
       <c r="B73" s="14" t="inlineStr">
         <is>
-          <t>test_ct_03_01_02_e_03_01_03_resumo_ate_500_palavras_e_ate_10_palavras_chave</t>
+          <t>test_ct_03_01_01_formulario_traz_turma_orientadores_e_areas</t>
         </is>
       </c>
       <c r="C73" s="14" t="n">
@@ -12019,7 +12019,7 @@
       </c>
       <c r="D73" s="14" t="inlineStr">
         <is>
-          <t>CT-03.01-02, CT-03.01-03</t>
+          <t>CT-03.01-01</t>
         </is>
       </c>
       <c r="E73" s="14" t="inlineStr">
@@ -12028,7 +12028,7 @@
         </is>
       </c>
       <c r="F73" s="14" t="n">
-        <v>1.647</v>
+        <v>1.903</v>
       </c>
       <c r="G73" s="14" t="inlineStr">
         <is>
@@ -12036,7 +12036,7 @@
         </is>
       </c>
       <c r="H73" s="14" t="n">
-        <v>2.052</v>
+        <v>1.804</v>
       </c>
     </row>
     <row r="74">
@@ -12047,7 +12047,7 @@
       </c>
       <c r="B74" s="14" t="inlineStr">
         <is>
-          <t>test_ct_03_01_04_e_03_04_02_e_06_01_01_rascunho_sem_protocolo_e_vinculo_pendente</t>
+          <t>test_ct_03_01_02_e_03_01_03_resumo_ate_500_palavras_e_ate_10_palavras_chave</t>
         </is>
       </c>
       <c r="C74" s="14" t="n">
@@ -12055,7 +12055,7 @@
       </c>
       <c r="D74" s="14" t="inlineStr">
         <is>
-          <t>CT-03.01-04, CT-03.01-05, CT-03.04-02, CT-06.01-01</t>
+          <t>CT-03.01-02, CT-03.01-03</t>
         </is>
       </c>
       <c r="E74" s="14" t="inlineStr">
@@ -12064,7 +12064,7 @@
         </is>
       </c>
       <c r="F74" s="14" t="n">
-        <v>1.901</v>
+        <v>1.852</v>
       </c>
       <c r="G74" s="14" t="inlineStr">
         <is>
@@ -12072,7 +12072,7 @@
         </is>
       </c>
       <c r="H74" s="14" t="n">
-        <v>2.198</v>
+        <v>1.849</v>
       </c>
     </row>
     <row r="75">
@@ -12083,7 +12083,7 @@
       </c>
       <c r="B75" s="14" t="inlineStr">
         <is>
-          <t>test_ct_03_01_08_editar_rascunho_audita_cada_campo</t>
+          <t>test_ct_03_01_04_e_03_04_02_e_06_01_01_rascunho_sem_protocolo_e_vinculo_pendente</t>
         </is>
       </c>
       <c r="C75" s="14" t="n">
@@ -12091,7 +12091,7 @@
       </c>
       <c r="D75" s="14" t="inlineStr">
         <is>
-          <t>CT-03.01-08</t>
+          <t>CT-03.01-04, CT-03.01-05, CT-03.04-02, CT-06.01-01</t>
         </is>
       </c>
       <c r="E75" s="14" t="inlineStr">
@@ -12100,7 +12100,7 @@
         </is>
       </c>
       <c r="F75" s="14" t="n">
-        <v>2.239</v>
+        <v>1.912</v>
       </c>
       <c r="G75" s="14" t="inlineStr">
         <is>
@@ -12108,7 +12108,7 @@
         </is>
       </c>
       <c r="H75" s="14" t="n">
-        <v>3.685</v>
+        <v>1.836</v>
       </c>
     </row>
     <row r="76">
@@ -12119,7 +12119,7 @@
       </c>
       <c r="B76" s="14" t="inlineStr">
         <is>
-          <t>test_ct_03_02_03_e_03_02_04_artigo_publicado_exige_doi</t>
+          <t>test_ct_03_01_08_editar_rascunho_audita_cada_campo</t>
         </is>
       </c>
       <c r="C76" s="14" t="n">
@@ -12127,7 +12127,7 @@
       </c>
       <c r="D76" s="14" t="inlineStr">
         <is>
-          <t>CT-03.02-03, CT-03.02-04</t>
+          <t>CT-03.01-08</t>
         </is>
       </c>
       <c r="E76" s="14" t="inlineStr">
@@ -12136,7 +12136,7 @@
         </is>
       </c>
       <c r="F76" s="14" t="n">
-        <v>2.236</v>
+        <v>1.992</v>
       </c>
       <c r="G76" s="14" t="inlineStr">
         <is>
@@ -12144,7 +12144,7 @@
         </is>
       </c>
       <c r="H76" s="14" t="n">
-        <v>3.65</v>
+        <v>2.117</v>
       </c>
     </row>
     <row r="77">
@@ -12155,7 +12155,7 @@
       </c>
       <c r="B77" s="14" t="inlineStr">
         <is>
-          <t>test_ct_03_03_01_e_03_03_06_e_03_04_01_submissao_gera_protocolo_unico_e_repetir_nao_duplica</t>
+          <t>test_ct_03_02_03_e_03_02_04_artigo_publicado_exige_doi</t>
         </is>
       </c>
       <c r="C77" s="14" t="n">
@@ -12163,7 +12163,7 @@
       </c>
       <c r="D77" s="14" t="inlineStr">
         <is>
-          <t>CT-03.03-01, CT-03.03-05, CT-03.03-06, CT-03.03-08, CT-03.04-01, CT-03.04-03, CT-03.04-06</t>
+          <t>CT-03.02-03, CT-03.02-04</t>
         </is>
       </c>
       <c r="E77" s="14" t="inlineStr">
@@ -12172,7 +12172,7 @@
         </is>
       </c>
       <c r="F77" s="14" t="n">
-        <v>2.427</v>
+        <v>2.041</v>
       </c>
       <c r="G77" s="14" t="inlineStr">
         <is>
@@ -12180,7 +12180,7 @@
         </is>
       </c>
       <c r="H77" s="14" t="n">
-        <v>2.276</v>
+        <v>1.819</v>
       </c>
     </row>
     <row r="78">
@@ -12191,7 +12191,7 @@
       </c>
       <c r="B78" s="14" t="inlineStr">
         <is>
-          <t>test_ct_03_03_02_campos_obrigatorios</t>
+          <t>test_ct_03_03_01_e_03_03_06_e_03_04_01_submissao_gera_protocolo_unico_e_repetir_nao_duplica</t>
         </is>
       </c>
       <c r="C78" s="14" t="n">
@@ -12199,7 +12199,7 @@
       </c>
       <c r="D78" s="14" t="inlineStr">
         <is>
-          <t>CT-03.03-02</t>
+          <t>CT-03.03-01, CT-03.03-05, CT-03.03-06, CT-03.03-08, CT-03.04-01, CT-03.04-03, CT-03.04-06</t>
         </is>
       </c>
       <c r="E78" s="14" t="inlineStr">
@@ -12208,7 +12208,7 @@
         </is>
       </c>
       <c r="F78" s="14" t="n">
-        <v>2.072</v>
+        <v>2.128</v>
       </c>
       <c r="G78" s="14" t="inlineStr">
         <is>
@@ -12216,7 +12216,7 @@
         </is>
       </c>
       <c r="H78" s="14" t="n">
-        <v>3.12</v>
+        <v>1.94</v>
       </c>
     </row>
     <row r="79">
@@ -12227,7 +12227,7 @@
       </c>
       <c r="B79" s="14" t="inlineStr">
         <is>
-          <t>test_ct_03_03_03_desistente_nao_submete</t>
+          <t>test_ct_03_03_02_campos_obrigatorios</t>
         </is>
       </c>
       <c r="C79" s="14" t="n">
@@ -12235,7 +12235,7 @@
       </c>
       <c r="D79" s="14" t="inlineStr">
         <is>
-          <t>CT-03.03-03</t>
+          <t>CT-03.03-02</t>
         </is>
       </c>
       <c r="E79" s="14" t="inlineStr">
@@ -12244,7 +12244,7 @@
         </is>
       </c>
       <c r="F79" s="14" t="n">
-        <v>2.039</v>
+        <v>2.007</v>
       </c>
       <c r="G79" s="14" t="inlineStr">
         <is>
@@ -12252,7 +12252,7 @@
         </is>
       </c>
       <c r="H79" s="14" t="n">
-        <v>3.813</v>
+        <v>1.969</v>
       </c>
     </row>
     <row r="80">
@@ -12263,7 +12263,7 @@
       </c>
       <c r="B80" s="14" t="inlineStr">
         <is>
-          <t>test_ct_03_04_04_um_cadastro_por_periodo</t>
+          <t>test_ct_03_03_03_desistente_nao_submete</t>
         </is>
       </c>
       <c r="C80" s="14" t="n">
@@ -12271,7 +12271,7 @@
       </c>
       <c r="D80" s="14" t="inlineStr">
         <is>
-          <t>CT-03.04-04</t>
+          <t>CT-03.03-03</t>
         </is>
       </c>
       <c r="E80" s="14" t="inlineStr">
@@ -12280,7 +12280,7 @@
         </is>
       </c>
       <c r="F80" s="14" t="n">
-        <v>1.939</v>
+        <v>2.052</v>
       </c>
       <c r="G80" s="14" t="inlineStr">
         <is>
@@ -12288,7 +12288,7 @@
         </is>
       </c>
       <c r="H80" s="14" t="n">
-        <v>2.243</v>
+        <v>4.178</v>
       </c>
     </row>
     <row r="81">
@@ -12299,7 +12299,7 @@
       </c>
       <c r="B81" s="14" t="inlineStr">
         <is>
-          <t>test_ds_fl01b_e2_orientador_nao_elegivel</t>
+          <t>test_ct_03_04_04_um_cadastro_por_periodo</t>
         </is>
       </c>
       <c r="C81" s="14" t="n">
@@ -12307,7 +12307,7 @@
       </c>
       <c r="D81" s="14" t="inlineStr">
         <is>
-          <t>complementar (sem CT na matriz)</t>
+          <t>CT-03.04-04</t>
         </is>
       </c>
       <c r="E81" s="14" t="inlineStr">
@@ -12316,7 +12316,7 @@
         </is>
       </c>
       <c r="F81" s="14" t="n">
-        <v>2.094</v>
+        <v>2.046</v>
       </c>
       <c r="G81" s="14" t="inlineStr">
         <is>
@@ -12324,7 +12324,7 @@
         </is>
       </c>
       <c r="H81" s="14" t="n">
-        <v>2.777</v>
+        <v>1.818</v>
       </c>
     </row>
     <row r="82">
@@ -12335,7 +12335,7 @@
       </c>
       <c r="B82" s="14" t="inlineStr">
         <is>
-          <t>test_ds_fl01b_em_analise_nao_edita</t>
+          <t>test_ds_fl01b_e2_orientador_nao_elegivel</t>
         </is>
       </c>
       <c r="C82" s="14" t="n">
@@ -12352,7 +12352,7 @@
         </is>
       </c>
       <c r="F82" s="14" t="n">
-        <v>2.022</v>
+        <v>1.818</v>
       </c>
       <c r="G82" s="14" t="inlineStr">
         <is>
@@ -12360,7 +12360,7 @@
         </is>
       </c>
       <c r="H82" s="14" t="n">
-        <v>3.563</v>
+        <v>1.756</v>
       </c>
     </row>
     <row r="83">
@@ -12371,7 +12371,7 @@
       </c>
       <c r="B83" s="14" t="inlineStr">
         <is>
-          <t>test_ds_fl03_orientador_aceita_e_aluno_e_avisado</t>
+          <t>test_ds_fl01b_em_analise_nao_edita</t>
         </is>
       </c>
       <c r="C83" s="14" t="n">
@@ -12388,7 +12388,7 @@
         </is>
       </c>
       <c r="F83" s="14" t="n">
-        <v>2.228</v>
+        <v>2.264</v>
       </c>
       <c r="G83" s="14" t="inlineStr">
         <is>
@@ -12396,7 +12396,7 @@
         </is>
       </c>
       <c r="H83" s="14" t="n">
-        <v>3.724</v>
+        <v>1.918</v>
       </c>
     </row>
     <row r="84">
@@ -12407,7 +12407,7 @@
       </c>
       <c r="B84" s="14" t="inlineStr">
         <is>
-          <t>test_ds_fl03_recusa_exige_motivo_e_nao_pode_responder_duas_vezes</t>
+          <t>test_ds_fl03_orientador_aceita_e_aluno_e_avisado</t>
         </is>
       </c>
       <c r="C84" s="14" t="n">
@@ -12424,7 +12424,7 @@
         </is>
       </c>
       <c r="F84" s="14" t="n">
-        <v>2.613</v>
+        <v>2.127</v>
       </c>
       <c r="G84" s="14" t="inlineStr">
         <is>
@@ -12432,7 +12432,7 @@
         </is>
       </c>
       <c r="H84" s="14" t="n">
-        <v>3.499</v>
+        <v>1.966</v>
       </c>
     </row>
     <row r="85">
@@ -12443,7 +12443,7 @@
       </c>
       <c r="B85" s="14" t="inlineStr">
         <is>
-          <t>test_ds_fl03b_apos_recusa_aluno_indica_outro_orientador</t>
+          <t>test_ds_fl03_recusa_exige_motivo_e_nao_pode_responder_duas_vezes</t>
         </is>
       </c>
       <c r="C85" s="14" t="n">
@@ -12460,7 +12460,7 @@
         </is>
       </c>
       <c r="F85" s="14" t="n">
-        <v>2.226</v>
+        <v>2.043</v>
       </c>
       <c r="G85" s="14" t="inlineStr">
         <is>
@@ -12468,7 +12468,7 @@
         </is>
       </c>
       <c r="H85" s="14" t="n">
-        <v>3.821</v>
+        <v>1.968</v>
       </c>
     </row>
     <row r="86">
@@ -12479,7 +12479,7 @@
       </c>
       <c r="B86" s="14" t="inlineStr">
         <is>
-          <t>test_minhas_turmas_do_aluno_mostra_matricula_e_o_proprio_tcc</t>
+          <t>test_ds_fl03b_apos_recusa_aluno_indica_outro_orientador</t>
         </is>
       </c>
       <c r="C86" s="14" t="n">
@@ -12496,7 +12496,7 @@
         </is>
       </c>
       <c r="F86" s="14" t="n">
-        <v>2.075</v>
+        <v>2.189</v>
       </c>
       <c r="G86" s="14" t="inlineStr">
         <is>
@@ -12504,7 +12504,7 @@
         </is>
       </c>
       <c r="H86" s="14" t="n">
-        <v>3.024</v>
+        <v>1.975</v>
       </c>
     </row>
     <row r="87">
@@ -12515,7 +12515,7 @@
       </c>
       <c r="B87" s="14" t="inlineStr">
         <is>
-          <t>test_minhas_turmas_do_professor_com_contagem_de_alunos_e_tccs</t>
+          <t>test_minhas_turmas_do_aluno_mostra_matricula_e_o_proprio_tcc</t>
         </is>
       </c>
       <c r="C87" s="14" t="n">
@@ -12532,7 +12532,7 @@
         </is>
       </c>
       <c r="F87" s="14" t="n">
-        <v>3.243</v>
+        <v>2.116</v>
       </c>
       <c r="G87" s="14" t="inlineStr">
         <is>
@@ -12540,7 +12540,7 @@
         </is>
       </c>
       <c r="H87" s="14" t="n">
-        <v>3.99</v>
+        <v>1.924</v>
       </c>
     </row>
     <row r="88">
@@ -12551,7 +12551,7 @@
       </c>
       <c r="B88" s="14" t="inlineStr">
         <is>
-          <t>test_minhas_turmas_so_mostra_ao_docente_as_turmas_que_ele_conduz</t>
+          <t>test_minhas_turmas_do_professor_com_contagem_de_alunos_e_tccs</t>
         </is>
       </c>
       <c r="C88" s="14" t="n">
@@ -12568,7 +12568,7 @@
         </is>
       </c>
       <c r="F88" s="14" t="n">
-        <v>2.342</v>
+        <v>2.411</v>
       </c>
       <c r="G88" s="14" t="inlineStr">
         <is>
@@ -12576,7 +12576,7 @@
         </is>
       </c>
       <c r="H88" s="14" t="n">
-        <v>3.284</v>
+        <v>2.275</v>
       </c>
     </row>
     <row r="89">
@@ -12587,7 +12587,7 @@
       </c>
       <c r="B89" s="14" t="inlineStr">
         <is>
-          <t>test_rbn0303_nao_submete_sem_aceite_do_orientador</t>
+          <t>test_minhas_turmas_so_mostra_ao_docente_as_turmas_que_ele_conduz</t>
         </is>
       </c>
       <c r="C89" s="14" t="n">
@@ -12604,7 +12604,7 @@
         </is>
       </c>
       <c r="F89" s="14" t="n">
-        <v>2.594</v>
+        <v>1.804</v>
       </c>
       <c r="G89" s="14" t="inlineStr">
         <is>
@@ -12612,7 +12612,7 @@
         </is>
       </c>
       <c r="H89" s="14" t="n">
-        <v>3.205</v>
+        <v>1.887</v>
       </c>
     </row>
     <row r="90">
@@ -12623,7 +12623,7 @@
       </c>
       <c r="B90" s="14" t="inlineStr">
         <is>
-          <t>test_rbn0305_devolvido_e_corrigido_mantem_o_protocolo</t>
+          <t>test_rbn0303_nao_submete_sem_aceite_do_orientador</t>
         </is>
       </c>
       <c r="C90" s="14" t="n">
@@ -12640,7 +12640,7 @@
         </is>
       </c>
       <c r="F90" s="14" t="n">
-        <v>2.352</v>
+        <v>1.977</v>
       </c>
       <c r="G90" s="14" t="inlineStr">
         <is>
@@ -12648,7 +12648,7 @@
         </is>
       </c>
       <c r="H90" s="14" t="n">
-        <v>4.102</v>
+        <v>1.887</v>
       </c>
     </row>
     <row r="91">
@@ -12659,7 +12659,7 @@
       </c>
       <c r="B91" s="14" t="inlineStr">
         <is>
-          <t>test_rbn0501_listas_por_perfil</t>
+          <t>test_rbn0305_devolvido_e_corrigido_mantem_o_protocolo</t>
         </is>
       </c>
       <c r="C91" s="14" t="n">
@@ -12676,7 +12676,7 @@
         </is>
       </c>
       <c r="F91" s="14" t="n">
-        <v>1.918</v>
+        <v>2.182</v>
       </c>
       <c r="G91" s="14" t="inlineStr">
         <is>
@@ -12684,7 +12684,7 @@
         </is>
       </c>
       <c r="H91" s="14" t="n">
-        <v>3.753</v>
+        <v>4.148</v>
       </c>
     </row>
     <row r="92">
@@ -12695,7 +12695,7 @@
       </c>
       <c r="B92" s="14" t="inlineStr">
         <is>
-          <t>test_rbn0801_so_a_coordenacao_cria_turma</t>
+          <t>test_rbn0501_listas_por_perfil</t>
         </is>
       </c>
       <c r="C92" s="14" t="n">
@@ -12712,7 +12712,7 @@
         </is>
       </c>
       <c r="F92" s="14" t="n">
-        <v>2.523</v>
+        <v>2.132</v>
       </c>
       <c r="G92" s="14" t="inlineStr">
         <is>
@@ -12720,7 +12720,7 @@
         </is>
       </c>
       <c r="H92" s="14" t="n">
-        <v>3.468</v>
+        <v>3.864</v>
       </c>
     </row>
     <row r="93">
@@ -12731,7 +12731,7 @@
       </c>
       <c r="B93" s="14" t="inlineStr">
         <is>
-          <t>test_rbn0801_turma_criada_com_codigo_do_curso_e_periodo</t>
+          <t>test_rbn0801_so_a_coordenacao_cria_turma</t>
         </is>
       </c>
       <c r="C93" s="14" t="n">
@@ -12748,7 +12748,7 @@
         </is>
       </c>
       <c r="F93" s="14" t="n">
-        <v>2.421</v>
+        <v>1.874</v>
       </c>
       <c r="G93" s="14" t="inlineStr">
         <is>
@@ -12756,7 +12756,7 @@
         </is>
       </c>
       <c r="H93" s="14" t="n">
-        <v>3.647</v>
+        <v>1.66</v>
       </c>
     </row>
     <row r="94">
@@ -12767,7 +12767,7 @@
       </c>
       <c r="B94" s="14" t="inlineStr">
         <is>
-          <t>test_rn05_aluno_sem_matricula_nao_abre_nem_salva</t>
+          <t>test_rbn0801_turma_criada_com_codigo_do_curso_e_periodo</t>
         </is>
       </c>
       <c r="C94" s="14" t="n">
@@ -12784,7 +12784,7 @@
         </is>
       </c>
       <c r="F94" s="14" t="n">
-        <v>2.321</v>
+        <v>2.114</v>
       </c>
       <c r="G94" s="14" t="inlineStr">
         <is>
@@ -12792,7 +12792,7 @@
         </is>
       </c>
       <c r="H94" s="14" t="n">
-        <v>2.312</v>
+        <v>1.713</v>
       </c>
     </row>
     <row r="95">
@@ -12803,7 +12803,7 @@
       </c>
       <c r="B95" s="14" t="inlineStr">
         <is>
-          <t>test_rn07_aluno_e_outro_docente_nao_abrem_a_turma</t>
+          <t>test_rn05_aluno_sem_matricula_nao_abre_nem_salva</t>
         </is>
       </c>
       <c r="C95" s="14" t="n">
@@ -12820,7 +12820,7 @@
         </is>
       </c>
       <c r="F95" s="14" t="n">
-        <v>2.192</v>
+        <v>2.316</v>
       </c>
       <c r="G95" s="14" t="inlineStr">
         <is>
@@ -12828,7 +12828,7 @@
         </is>
       </c>
       <c r="H95" s="14" t="n">
-        <v>2.257</v>
+        <v>2.099</v>
       </c>
     </row>
     <row r="96">
@@ -12839,7 +12839,7 @@
       </c>
       <c r="B96" s="14" t="inlineStr">
         <is>
-          <t>test_rn07_orientador_so_responde_os_proprios_pedidos</t>
+          <t>test_rn07_aluno_e_outro_docente_nao_abrem_a_turma</t>
         </is>
       </c>
       <c r="C96" s="14" t="n">
@@ -12856,7 +12856,7 @@
         </is>
       </c>
       <c r="F96" s="14" t="n">
-        <v>2.141</v>
+        <v>1.809</v>
       </c>
       <c r="G96" s="14" t="inlineStr">
         <is>
@@ -12864,7 +12864,7 @@
         </is>
       </c>
       <c r="H96" s="14" t="n">
-        <v>4.23</v>
+        <v>1.794</v>
       </c>
     </row>
     <row r="97">
@@ -12875,7 +12875,7 @@
       </c>
       <c r="B97" s="14" t="inlineStr">
         <is>
-          <t>test_rn07_outro_aluno_nao_ve_nem_edita</t>
+          <t>test_rn07_orientador_so_responde_os_proprios_pedidos</t>
         </is>
       </c>
       <c r="C97" s="14" t="n">
@@ -12892,7 +12892,7 @@
         </is>
       </c>
       <c r="F97" s="14" t="n">
-        <v>2.849</v>
+        <v>1.947</v>
       </c>
       <c r="G97" s="14" t="inlineStr">
         <is>
@@ -12900,18 +12900,18 @@
         </is>
       </c>
       <c r="H97" s="14" t="n">
-        <v>4.547</v>
+        <v>1.855</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="14" t="inlineStr">
         <is>
-          <t>test_usuarios.py</t>
+          <t>test_tcc.py</t>
         </is>
       </c>
       <c r="B98" s="14" t="inlineStr">
         <is>
-          <t>test_ct_01_01_01_docente_nasce_inativo_e_sem_senha</t>
+          <t>test_rn07_outro_aluno_nao_ve_nem_edita</t>
         </is>
       </c>
       <c r="C98" s="14" t="n">
@@ -12919,7 +12919,7 @@
       </c>
       <c r="D98" s="14" t="inlineStr">
         <is>
-          <t>CT-01.01-01</t>
+          <t>complementar (sem CT na matriz)</t>
         </is>
       </c>
       <c r="E98" s="14" t="inlineStr">
@@ -12928,7 +12928,7 @@
         </is>
       </c>
       <c r="F98" s="14" t="n">
-        <v>0.806</v>
+        <v>2.287</v>
       </c>
       <c r="G98" s="14" t="inlineStr">
         <is>
@@ -12936,7 +12936,7 @@
         </is>
       </c>
       <c r="H98" s="14" t="n">
-        <v>1.54</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="99">
@@ -12947,7 +12947,7 @@
       </c>
       <c r="B99" s="14" t="inlineStr">
         <is>
-          <t>test_ct_01_01_02_campo_obrigatorio_vazio_responde_400</t>
+          <t>test_ct_01_01_01_docente_nasce_inativo_e_sem_senha</t>
         </is>
       </c>
       <c r="C99" s="14" t="n">
@@ -12955,7 +12955,7 @@
       </c>
       <c r="D99" s="14" t="inlineStr">
         <is>
-          <t>CT-01.01-02</t>
+          <t>CT-01.01-01</t>
         </is>
       </c>
       <c r="E99" s="14" t="inlineStr">
@@ -12964,7 +12964,7 @@
         </is>
       </c>
       <c r="F99" s="14" t="n">
-        <v>0.799</v>
+        <v>0.8120000000000001</v>
       </c>
       <c r="G99" s="14" t="inlineStr">
         <is>
@@ -12972,7 +12972,7 @@
         </is>
       </c>
       <c r="H99" s="14" t="n">
-        <v>1.04</v>
+        <v>2.131</v>
       </c>
     </row>
     <row r="100">
@@ -12983,7 +12983,7 @@
       </c>
       <c r="B100" s="14" t="inlineStr">
         <is>
-          <t>test_ct_01_01_03_email_duplicado_ignora_maiusculas</t>
+          <t>test_ct_01_01_02_campo_obrigatorio_vazio_responde_400</t>
         </is>
       </c>
       <c r="C100" s="14" t="n">
@@ -12991,7 +12991,7 @@
       </c>
       <c r="D100" s="14" t="inlineStr">
         <is>
-          <t>CT-01.01-03</t>
+          <t>CT-01.01-02</t>
         </is>
       </c>
       <c r="E100" s="14" t="inlineStr">
@@ -13000,7 +13000,7 @@
         </is>
       </c>
       <c r="F100" s="14" t="n">
-        <v>0.994</v>
+        <v>0.786</v>
       </c>
       <c r="G100" s="14" t="inlineStr">
         <is>
@@ -13008,7 +13008,7 @@
         </is>
       </c>
       <c r="H100" s="14" t="n">
-        <v>1.175</v>
+        <v>1.096</v>
       </c>
     </row>
     <row r="101">
@@ -13019,7 +13019,7 @@
       </c>
       <c r="B101" s="14" t="inlineStr">
         <is>
-          <t>test_ct_01_01_05_coordenador_nao_exige_curso</t>
+          <t>test_ct_01_01_03_email_duplicado_ignora_maiusculas</t>
         </is>
       </c>
       <c r="C101" s="14" t="n">
@@ -13027,7 +13027,7 @@
       </c>
       <c r="D101" s="14" t="inlineStr">
         <is>
-          <t>CT-01.01-05</t>
+          <t>CT-01.01-03</t>
         </is>
       </c>
       <c r="E101" s="14" t="inlineStr">
@@ -13036,7 +13036,7 @@
         </is>
       </c>
       <c r="F101" s="14" t="n">
-        <v>0.843</v>
+        <v>0.837</v>
       </c>
       <c r="G101" s="14" t="inlineStr">
         <is>
@@ -13044,7 +13044,7 @@
         </is>
       </c>
       <c r="H101" s="14" t="n">
-        <v>1.382</v>
+        <v>1.91</v>
       </c>
     </row>
     <row r="102">
@@ -13055,7 +13055,7 @@
       </c>
       <c r="B102" s="14" t="inlineStr">
         <is>
-          <t>test_ct_01_01_06_quem_nao_e_coordenador_recebe_403</t>
+          <t>test_ct_01_01_05_coordenador_nao_exige_curso</t>
         </is>
       </c>
       <c r="C102" s="14" t="n">
@@ -13063,7 +13063,7 @@
       </c>
       <c r="D102" s="14" t="inlineStr">
         <is>
-          <t>CT-01.01-06</t>
+          <t>CT-01.01-05</t>
         </is>
       </c>
       <c r="E102" s="14" t="inlineStr">
@@ -13072,7 +13072,7 @@
         </is>
       </c>
       <c r="F102" s="14" t="n">
-        <v>1.102</v>
+        <v>0.868</v>
       </c>
       <c r="G102" s="14" t="inlineStr">
         <is>
@@ -13080,7 +13080,7 @@
         </is>
       </c>
       <c r="H102" s="14" t="n">
-        <v>1.96</v>
+        <v>1.919</v>
       </c>
     </row>
     <row r="103">
@@ -13091,7 +13091,7 @@
       </c>
       <c r="B103" s="14" t="inlineStr">
         <is>
-          <t>test_ct_01_01_07_criacao_fica_no_log</t>
+          <t>test_ct_01_01_06_quem_nao_e_coordenador_recebe_403</t>
         </is>
       </c>
       <c r="C103" s="14" t="n">
@@ -13099,7 +13099,7 @@
       </c>
       <c r="D103" s="14" t="inlineStr">
         <is>
-          <t>CT-01.01-07</t>
+          <t>CT-01.01-06</t>
         </is>
       </c>
       <c r="E103" s="14" t="inlineStr">
@@ -13108,7 +13108,7 @@
         </is>
       </c>
       <c r="F103" s="14" t="n">
-        <v>0.854</v>
+        <v>1.128</v>
       </c>
       <c r="G103" s="14" t="inlineStr">
         <is>
@@ -13116,7 +13116,7 @@
         </is>
       </c>
       <c r="H103" s="14" t="n">
-        <v>1.489</v>
+        <v>1.88</v>
       </c>
     </row>
     <row r="104">
@@ -13127,7 +13127,7 @@
       </c>
       <c r="B104" s="14" t="inlineStr">
         <is>
-          <t>test_ct_01_03_01_aluno_nasce_sem_senha_com_perfil_aluno</t>
+          <t>test_ct_01_01_07_criacao_fica_no_log</t>
         </is>
       </c>
       <c r="C104" s="14" t="n">
@@ -13135,7 +13135,7 @@
       </c>
       <c r="D104" s="14" t="inlineStr">
         <is>
-          <t>CT-01.03-01</t>
+          <t>CT-01.01-07</t>
         </is>
       </c>
       <c r="E104" s="14" t="inlineStr">
@@ -13144,7 +13144,7 @@
         </is>
       </c>
       <c r="F104" s="14" t="n">
-        <v>1.155</v>
+        <v>1.034</v>
       </c>
       <c r="G104" s="14" t="inlineStr">
         <is>
@@ -13152,7 +13152,7 @@
         </is>
       </c>
       <c r="H104" s="14" t="n">
-        <v>1.055</v>
+        <v>1.239</v>
       </c>
     </row>
     <row r="105">
@@ -13163,7 +13163,7 @@
       </c>
       <c r="B105" s="14" t="inlineStr">
         <is>
-          <t>test_ct_01_03_03_indica_o_campo_duplicado</t>
+          <t>test_ct_01_03_01_aluno_nasce_sem_senha_com_perfil_aluno</t>
         </is>
       </c>
       <c r="C105" s="14" t="n">
@@ -13171,7 +13171,7 @@
       </c>
       <c r="D105" s="14" t="inlineStr">
         <is>
-          <t>CT-01.03-03</t>
+          <t>CT-01.03-01</t>
         </is>
       </c>
       <c r="E105" s="14" t="inlineStr">
@@ -13180,7 +13180,7 @@
         </is>
       </c>
       <c r="F105" s="14" t="n">
-        <v>0.878</v>
+        <v>0.823</v>
       </c>
       <c r="G105" s="14" t="inlineStr">
         <is>
@@ -13188,7 +13188,7 @@
         </is>
       </c>
       <c r="H105" s="14" t="n">
-        <v>1.447</v>
+        <v>1.074</v>
       </c>
     </row>
     <row r="106">
@@ -13199,7 +13199,7 @@
       </c>
       <c r="B106" s="14" t="inlineStr">
         <is>
-          <t>test_ct_01_03_06_e_01_05_01_enfileira_ativacao_e_audita</t>
+          <t>test_ct_01_03_03_indica_o_campo_duplicado</t>
         </is>
       </c>
       <c r="C106" s="14" t="n">
@@ -13207,7 +13207,7 @@
       </c>
       <c r="D106" s="14" t="inlineStr">
         <is>
-          <t>CT-01.03-06, CT-01.05-01</t>
+          <t>CT-01.03-03</t>
         </is>
       </c>
       <c r="E106" s="14" t="inlineStr">
@@ -13216,7 +13216,7 @@
         </is>
       </c>
       <c r="F106" s="14" t="n">
-        <v>0.833</v>
+        <v>0.875</v>
       </c>
       <c r="G106" s="14" t="inlineStr">
         <is>
@@ -13224,7 +13224,7 @@
         </is>
       </c>
       <c r="H106" s="14" t="n">
-        <v>1.407</v>
+        <v>1.822</v>
       </c>
     </row>
     <row r="107">
@@ -13235,7 +13235,7 @@
       </c>
       <c r="B107" s="14" t="inlineStr">
         <is>
-          <t>test_ct_01_08_01_e_01_08_06_edicao_auditada_com_valor_anterior_e_novo</t>
+          <t>test_ct_01_03_06_e_01_05_01_enfileira_ativacao_e_audita</t>
         </is>
       </c>
       <c r="C107" s="14" t="n">
@@ -13243,7 +13243,7 @@
       </c>
       <c r="D107" s="14" t="inlineStr">
         <is>
-          <t>CT-01.08-01, CT-01.08-06</t>
+          <t>CT-01.03-06, CT-01.05-01</t>
         </is>
       </c>
       <c r="E107" s="14" t="inlineStr">
@@ -13252,7 +13252,7 @@
         </is>
       </c>
       <c r="F107" s="14" t="n">
-        <v>0.923</v>
+        <v>0.829</v>
       </c>
       <c r="G107" s="14" t="inlineStr">
         <is>
@@ -13260,7 +13260,7 @@
         </is>
       </c>
       <c r="H107" s="14" t="n">
-        <v>1.17</v>
+        <v>1.543</v>
       </c>
     </row>
     <row r="108">
@@ -13271,7 +13271,7 @@
       </c>
       <c r="B108" s="14" t="inlineStr">
         <is>
-          <t>test_ct_01_08_02_email_ou_matricula_de_outra_pessoa</t>
+          <t>test_ct_01_08_01_e_01_08_06_edicao_auditada_com_valor_anterior_e_novo</t>
         </is>
       </c>
       <c r="C108" s="14" t="n">
@@ -13279,7 +13279,7 @@
       </c>
       <c r="D108" s="14" t="inlineStr">
         <is>
-          <t>CT-01.08-02</t>
+          <t>CT-01.08-01, CT-01.08-06</t>
         </is>
       </c>
       <c r="E108" s="14" t="inlineStr">
@@ -13288,7 +13288,7 @@
         </is>
       </c>
       <c r="F108" s="14" t="n">
-        <v>0.907</v>
+        <v>0.885</v>
       </c>
       <c r="G108" s="14" t="inlineStr">
         <is>
@@ -13296,7 +13296,7 @@
         </is>
       </c>
       <c r="H108" s="14" t="n">
-        <v>1.346</v>
+        <v>1.394</v>
       </c>
     </row>
     <row r="109">
@@ -13307,7 +13307,7 @@
       </c>
       <c r="B109" s="14" t="inlineStr">
         <is>
-          <t>test_ct_01_08_03_e_01_08_04_inativado_nao_entra_e_reativado_volta</t>
+          <t>test_ct_01_08_02_email_ou_matricula_de_outra_pessoa</t>
         </is>
       </c>
       <c r="C109" s="14" t="n">
@@ -13315,7 +13315,7 @@
       </c>
       <c r="D109" s="14" t="inlineStr">
         <is>
-          <t>CT-01.06-08, CT-01.08-03, CT-01.08-04</t>
+          <t>CT-01.08-02</t>
         </is>
       </c>
       <c r="E109" s="14" t="inlineStr">
@@ -13324,7 +13324,7 @@
         </is>
       </c>
       <c r="F109" s="14" t="n">
-        <v>1.389</v>
+        <v>0.896</v>
       </c>
       <c r="G109" s="14" t="inlineStr">
         <is>
@@ -13332,7 +13332,7 @@
         </is>
       </c>
       <c r="H109" s="14" t="n">
-        <v>2.326</v>
+        <v>1.296</v>
       </c>
     </row>
     <row r="110">
@@ -13343,7 +13343,7 @@
       </c>
       <c r="B110" s="14" t="inlineStr">
         <is>
-          <t>test_hu0101_ca6_ninguem_altera_os_proprios_perfis</t>
+          <t>test_ct_01_08_03_e_01_08_04_inativado_nao_entra_e_reativado_volta</t>
         </is>
       </c>
       <c r="C110" s="14" t="n">
@@ -13351,7 +13351,7 @@
       </c>
       <c r="D110" s="14" t="inlineStr">
         <is>
-          <t>complementar (sem CT na matriz)</t>
+          <t>CT-01.06-08, CT-01.08-03, CT-01.08-04</t>
         </is>
       </c>
       <c r="E110" s="14" t="inlineStr">
@@ -13360,7 +13360,7 @@
         </is>
       </c>
       <c r="F110" s="14" t="n">
-        <v>1.012</v>
+        <v>1.395</v>
       </c>
       <c r="G110" s="14" t="inlineStr">
         <is>
@@ -13368,7 +13368,7 @@
         </is>
       </c>
       <c r="H110" s="14" t="n">
-        <v>2.056</v>
+        <v>2.765</v>
       </c>
     </row>
     <row r="111">
@@ -13379,7 +13379,7 @@
       </c>
       <c r="B111" s="14" t="inlineStr">
         <is>
-          <t>test_hu0103_busca_e_filtro_por_curso</t>
+          <t>test_hu0101_ca6_ninguem_altera_os_proprios_perfis</t>
         </is>
       </c>
       <c r="C111" s="14" t="n">
@@ -13396,7 +13396,7 @@
         </is>
       </c>
       <c r="F111" s="14" t="n">
-        <v>0.976</v>
+        <v>1.162</v>
       </c>
       <c r="G111" s="14" t="inlineStr">
         <is>
@@ -13404,7 +13404,7 @@
         </is>
       </c>
       <c r="H111" s="14" t="n">
-        <v>1.325</v>
+        <v>1.946</v>
       </c>
     </row>
     <row r="112">
@@ -13415,7 +13415,7 @@
       </c>
       <c r="B112" s="14" t="inlineStr">
         <is>
-          <t>test_hu0103_e1_curso_fora_dos_contemplados</t>
+          <t>test_hu0103_busca_e_filtro_por_curso</t>
         </is>
       </c>
       <c r="C112" s="14" t="n">
@@ -13432,7 +13432,7 @@
         </is>
       </c>
       <c r="F112" s="14" t="n">
-        <v>1.028</v>
+        <v>0.982</v>
       </c>
       <c r="G112" s="14" t="inlineStr">
         <is>
@@ -13440,7 +13440,7 @@
         </is>
       </c>
       <c r="H112" s="14" t="n">
-        <v>1.016</v>
+        <v>1.599</v>
       </c>
     </row>
     <row r="113">
@@ -13451,7 +13451,7 @@
       </c>
       <c r="B113" s="14" t="inlineStr">
         <is>
-          <t>test_hu0108_ca4_nao_existe_rota_de_exclusao</t>
+          <t>test_hu0103_e1_curso_fora_dos_contemplados</t>
         </is>
       </c>
       <c r="C113" s="14" t="n">
@@ -13468,7 +13468,7 @@
         </is>
       </c>
       <c r="F113" s="14" t="n">
-        <v>0.823</v>
+        <v>0.986</v>
       </c>
       <c r="G113" s="14" t="inlineStr">
         <is>
@@ -13476,7 +13476,7 @@
         </is>
       </c>
       <c r="H113" s="14" t="n">
-        <v>1.386</v>
+        <v>1.355</v>
       </c>
     </row>
     <row r="114">
@@ -13487,7 +13487,7 @@
       </c>
       <c r="B114" s="14" t="inlineStr">
         <is>
-          <t>test_hu0108_coordenador_nao_inativa_a_si_mesmo</t>
+          <t>test_hu0108_ca4_nao_existe_rota_de_exclusao</t>
         </is>
       </c>
       <c r="C114" s="14" t="n">
@@ -13504,7 +13504,7 @@
         </is>
       </c>
       <c r="F114" s="14" t="n">
-        <v>0.8149999999999999</v>
+        <v>1.076</v>
       </c>
       <c r="G114" s="14" t="inlineStr">
         <is>
@@ -13512,12 +13512,48 @@
         </is>
       </c>
       <c r="H114" s="14" t="n">
-        <v>1.54</v>
+        <v>1.273</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="14" t="inlineStr">
+        <is>
+          <t>test_usuarios.py</t>
+        </is>
+      </c>
+      <c r="B115" s="14" t="inlineStr">
+        <is>
+          <t>test_hu0108_coordenador_nao_inativa_a_si_mesmo</t>
+        </is>
+      </c>
+      <c r="C115" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D115" s="14" t="inlineStr">
+        <is>
+          <t>complementar (sem CT na matriz)</t>
+        </is>
+      </c>
+      <c r="E115" s="14" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="F115" s="14" t="n">
+        <v>0.826</v>
+      </c>
+      <c r="G115" s="14" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="H115" s="14" t="n">
+        <v>1.057</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H114"/>
-  <conditionalFormatting sqref="E2:E114">
+  <autoFilter ref="A1:H115"/>
+  <conditionalFormatting sqref="E2:E115">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$E2="Aprovado"</formula>
     </cfRule>
@@ -13534,7 +13570,7 @@
       <formula>$E2="Pulado"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G114">
+  <conditionalFormatting sqref="G2:G115">
     <cfRule type="expression" priority="6" dxfId="0">
       <formula>$G2="Aprovado"</formula>
     </cfRule>

</xml_diff>